<commit_message>
WIP：每小时保存全部进度 2026-09-18 03:56:32 -04:00
</commit_message>
<xml_diff>
--- a/data/tip/Tip.xlsx
+++ b/data/tip/Tip.xlsx
@@ -1020,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C261"/>
+  <dimension ref="A1:C270"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="8" customWidth="1" style="2" min="3" max="3"/>
@@ -2911,833 +2911,941 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="0" t="inlineStr">
-        <is>
-          <t>//friend_error base=15000 width=1000</t>
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>GuildZoneMerging</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>区服合并维护中，帮会操作暂停，请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="0" t="inlineStr">
-        <is>
-          <t>FriendCannotAddSelf</t>
-        </is>
-      </c>
-      <c r="B188" s="0" t="inlineStr">
-        <is>
-          <t>不能添加自己为好友</t>
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>GuildTargetNotMember</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>对方已不在本帮会</t>
         </is>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="0" t="inlineStr">
-        <is>
-          <t>FriendAlreadyFriends</t>
-        </is>
-      </c>
-      <c r="B189" s="0" t="inlineStr">
-        <is>
-          <t>你们已经是好友了</t>
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>GuildCannotTargetSelf</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>不能对自己执行此操作</t>
         </is>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="0" t="inlineStr">
-        <is>
-          <t>FriendListFull</t>
-        </is>
-      </c>
-      <c r="B190" s="0" t="inlineStr">
-        <is>
-          <t>好友列表已满</t>
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>GuildRankTooLow</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>帮会职位不足，无法执行此操作</t>
         </is>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="0" t="inlineStr">
-        <is>
-          <t>FriendRequestAlreadySent</t>
-        </is>
-      </c>
-      <c r="B191" s="0" t="inlineStr">
-        <is>
-          <t>已发送过好友申请</t>
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>GuildOfficerLimit</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>长老人数已达当前帮会等级上限</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="0" t="inlineStr">
-        <is>
-          <t>FriendTargetListFull</t>
-        </is>
-      </c>
-      <c r="B192" s="0" t="inlineStr">
-        <is>
-          <t>对方好友列表已满</t>
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>GuildApplicationNotFound</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>入帮申请不存在或已失效</t>
         </is>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="0" t="inlineStr">
-        <is>
-          <t>FriendNoPendingRequest</t>
-        </is>
-      </c>
-      <c r="B193" s="0" t="inlineStr">
-        <is>
-          <t>没有待处理的好友申请</t>
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>GuildApplicationLimit</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>同时进行中的入帮申请已达上限</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="0" t="inlineStr">
-        <is>
-          <t>FriendTooManyPending</t>
-        </is>
-      </c>
-      <c r="B194" s="0" t="inlineStr">
-        <is>
-          <t>待处理的申请过多</t>
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>GuildApplicationQueueFull</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>该帮会待审申请已满，请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="0" t="inlineStr">
-        <is>
-          <t>//match_error base=16000 width=1000</t>
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>GuildBusyRetry</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>帮会操作繁忙，请稍后重试</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t>MatchInBattle</t>
-        </is>
-      </c>
-      <c r="B196" s="0" t="inlineStr">
-        <is>
-          <t>你正在战斗中</t>
+          <t>//friend_error base=15000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t>MatchAlreadyQueued</t>
+          <t>FriendCannotAddSelf</t>
         </is>
       </c>
       <c r="B197" s="0" t="inlineStr">
         <is>
-          <t>已在匹配队列中</t>
+          <t>不能添加自己为好友</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t>MatchModeNotOpen</t>
+          <t>FriendAlreadyFriends</t>
         </is>
       </c>
       <c r="B198" s="0" t="inlineStr">
         <is>
-          <t>该匹配模式暂未开放</t>
+          <t>你们已经是好友了</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t>MatchTeamSizeNotConfigured</t>
+          <t>FriendListFull</t>
         </is>
       </c>
       <c r="B199" s="0" t="inlineStr">
         <is>
-          <t>队伍人数未配置</t>
+          <t>好友列表已满</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t>MatchInternal</t>
+          <t>FriendRequestAlreadySent</t>
         </is>
       </c>
       <c r="B200" s="0" t="inlineStr">
         <is>
-          <t>服务繁忙，请稍后重试</t>
-        </is>
-      </c>
-      <c r="C200" s="0" t="n"/>
+          <t>已发送过好友申请</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t>MatchTicketMismatch</t>
+          <t>FriendTargetListFull</t>
         </is>
       </c>
       <c r="B201" s="0" t="inlineStr">
         <is>
-          <t>匹配凭据不匹配</t>
+          <t>对方好友列表已满</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t>MatchCancelTooLate</t>
+          <t>FriendNoPendingRequest</t>
         </is>
       </c>
       <c r="B202" s="0" t="inlineStr">
         <is>
-          <t>匹配已开始，无法取消</t>
+          <t>没有待处理的好友申请</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeSelf</t>
+          <t>FriendTooManyPending</t>
         </is>
       </c>
       <c r="B203" s="0" t="inlineStr">
         <is>
-          <t>不能挑战自己</t>
+          <t>待处理的申请过多</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeTargetOffline</t>
-        </is>
-      </c>
-      <c r="B204" s="0" t="inlineStr">
-        <is>
-          <t>对方不在线</t>
+          <t>//match_error base=16000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeTargetBusy</t>
+          <t>MatchInBattle</t>
         </is>
       </c>
       <c r="B205" s="0" t="inlineStr">
         <is>
-          <t>对方正在战斗中</t>
+          <t>你正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeSelfBusy</t>
+          <t>MatchAlreadyQueued</t>
         </is>
       </c>
       <c r="B206" s="0" t="inlineStr">
         <is>
-          <t>你正在战斗中</t>
+          <t>已在匹配队列中</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengePending</t>
+          <t>MatchModeNotOpen</t>
         </is>
       </c>
       <c r="B207" s="0" t="inlineStr">
         <is>
-          <t>已有待应答的挑战</t>
+          <t>该匹配模式暂未开放</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeExpired</t>
+          <t>MatchTeamSizeNotConfigured</t>
         </is>
       </c>
       <c r="B208" s="0" t="inlineStr">
         <is>
-          <t>挑战已过期</t>
+          <t>队伍人数未配置</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeNotTarget</t>
+          <t>MatchInternal</t>
         </is>
       </c>
       <c r="B209" s="0" t="inlineStr">
         <is>
-          <t>你不是该挑战的对象</t>
-        </is>
-      </c>
+          <t>服务繁忙，请稍后重试</t>
+        </is>
+      </c>
+      <c r="C209" s="0" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateWhileQueued</t>
+          <t>MatchTicketMismatch</t>
         </is>
       </c>
       <c r="B210" s="0" t="inlineStr">
         <is>
-          <t>匹配中无法观战</t>
+          <t>匹配凭据不匹配</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateWhileInBattle</t>
+          <t>MatchCancelTooLate</t>
         </is>
       </c>
       <c r="B211" s="0" t="inlineStr">
         <is>
-          <t>战斗中无法观战</t>
+          <t>匹配已开始，无法取消</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t>MatchAlreadyWatching</t>
+          <t>MatchChallengeSelf</t>
         </is>
       </c>
       <c r="B212" s="0" t="inlineStr">
         <is>
-          <t>已在观战中</t>
+          <t>不能挑战自己</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t>MatchNoWatchableBattle</t>
+          <t>MatchChallengeTargetOffline</t>
         </is>
       </c>
       <c r="B213" s="0" t="inlineStr">
         <is>
-          <t>当前没有可观战的战斗</t>
+          <t>对方不在线</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t>MatchBattleNotWatchable</t>
+          <t>MatchChallengeTargetBusy</t>
         </is>
       </c>
       <c r="B214" s="0" t="inlineStr">
         <is>
-          <t>该战斗无法观战</t>
+          <t>对方正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateOffline</t>
+          <t>MatchChallengeSelfBusy</t>
         </is>
       </c>
       <c r="B215" s="0" t="inlineStr">
         <is>
-          <t>观战会话已断开</t>
+          <t>你正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t>MatchNotInScene</t>
+          <t>MatchChallengePending</t>
         </is>
       </c>
       <c r="B216" s="0" t="inlineStr">
         <is>
-          <t>请先进入场景</t>
+          <t>已有待应答的挑战</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t>// 以下号段为移植域预留，建组时把本行改成组头即可：</t>
+          <t>MatchChallengeExpired</t>
+        </is>
+      </c>
+      <c r="B217" s="0" t="inlineStr">
+        <is>
+          <t>挑战已过期</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t>//   mail_error 17000 / chat_error 18000 / auction_error 19000</t>
+          <t>MatchChallengeNotTarget</t>
+        </is>
+      </c>
+      <c r="B218" s="0" t="inlineStr">
+        <is>
+          <t>你不是该挑战的对象</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t>//   rank_error 21000 / dialogue_error 22000 / battle_result_error 23000 / grant_error 24000</t>
-        </is>
-      </c>
-    </row>
-    <row r="220"/>
+          <t>MatchSpectateWhileQueued</t>
+        </is>
+      </c>
+      <c r="B219" s="0" t="inlineStr">
+        <is>
+          <t>匹配中无法观战</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="0" t="inlineStr">
+        <is>
+          <t>MatchSpectateWhileInBattle</t>
+        </is>
+      </c>
+      <c r="B220" s="0" t="inlineStr">
+        <is>
+          <t>战斗中无法观战</t>
+        </is>
+      </c>
+    </row>
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t>//trade_error base=20000 width=1000</t>
+          <t>MatchAlreadyWatching</t>
+        </is>
+      </c>
+      <c r="B221" s="0" t="inlineStr">
+        <is>
+          <t>已在观战中</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t>TradeListingNotFound</t>
+          <t>MatchNoWatchableBattle</t>
         </is>
       </c>
       <c r="B222" s="0" t="inlineStr">
         <is>
-          <t>商品不存在或已下架</t>
+          <t>当前没有可观战的战斗</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t>TradeHomeZoneUnknown</t>
+          <t>MatchBattleNotWatchable</t>
         </is>
       </c>
       <c r="B223" s="0" t="inlineStr">
         <is>
-          <t>角色归属区服未确认，暂时无法使用聚宝斋</t>
+          <t>该战斗无法观战</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t>TradeFavoriteLimitReached</t>
+          <t>MatchSpectateOffline</t>
         </is>
       </c>
       <c r="B224" s="0" t="inlineStr">
         <is>
-          <t>收藏数量已达上限，请先取消部分收藏</t>
+          <t>观战会话已断开</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t>TradeFeatureDisabled</t>
+          <t>MatchNotInScene</t>
         </is>
       </c>
       <c r="B225" s="0" t="inlineStr">
         <is>
-          <t>该功能尚未开放</t>
-        </is>
-      </c>
-    </row>
-    <row r="226"/>
+          <t>请先进入场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="0" t="inlineStr">
+        <is>
+          <t>// 以下号段为移植域预留，建组时把本行改成组头即可：</t>
+        </is>
+      </c>
+    </row>
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t>//attribute_error base=25000 width=1000</t>
+          <t>//   mail_error 17000 / chat_error 18000 / auction_error 19000</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t>AttributePoolNotFound</t>
-        </is>
-      </c>
-      <c r="B228" s="0" t="inlineStr">
-        <is>
-          <t>属性池不存在</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" s="0" t="inlineStr">
-        <is>
-          <t>AttributePoolLocked</t>
-        </is>
-      </c>
-      <c r="B229" s="0" t="inlineStr">
-        <is>
-          <t>该属性池尚未解锁</t>
-        </is>
-      </c>
-    </row>
+          <t>//   rank_error 21000 / dialogue_error 22000 / battle_result_error 23000 / grant_error 24000</t>
+        </is>
+      </c>
+    </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t>AttributeDimensionNotFound</t>
-        </is>
-      </c>
-      <c r="B230" s="0" t="inlineStr">
-        <is>
-          <t>属性维度不存在</t>
+          <t>//trade_error base=20000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t>AttributePointsNotEnough</t>
+          <t>TradeListingNotFound</t>
         </is>
       </c>
       <c r="B231" s="0" t="inlineStr">
         <is>
-          <t>剩余点数不足</t>
+          <t>商品不存在或已下架</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t>AttributePointsCannotDecrease</t>
+          <t>TradeHomeZoneUnknown</t>
         </is>
       </c>
       <c r="B232" s="0" t="inlineStr">
         <is>
-          <t>已分配的点数不能减少,请使用重置</t>
+          <t>角色归属区服未确认，暂时无法使用聚宝斋</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t>AttributeDimensionCapExceeded</t>
+          <t>TradeFavoriteLimitReached</t>
         </is>
       </c>
       <c r="B233" s="0" t="inlineStr">
         <is>
-          <t>超过单项可分配上限</t>
+          <t>收藏数量已达上限，请先取消部分收藏</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeNotFound</t>
+          <t>TradeFeatureDisabled</t>
         </is>
       </c>
       <c r="B234" s="0" t="inlineStr">
         <is>
-          <t>加点方案不存在</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" s="0" t="inlineStr">
-        <is>
-          <t>AttributeSchemeLimitReached</t>
-        </is>
-      </c>
-      <c r="B235" s="0" t="inlineStr">
-        <is>
-          <t>加点方案数量已达上限</t>
-        </is>
-      </c>
-    </row>
+          <t>该功能尚未开放</t>
+        </is>
+      </c>
+    </row>
+    <row r="235"/>
     <row r="236">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeSwitchCooldown</t>
-        </is>
-      </c>
-      <c r="B236" s="0" t="inlineStr">
-        <is>
-          <t>方案切换冷却中</t>
+          <t>//attribute_error base=25000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeNameInvalid</t>
+          <t>AttributePoolNotFound</t>
         </is>
       </c>
       <c r="B237" s="0" t="inlineStr">
         <is>
-          <t>方案名称不合法</t>
+          <t>属性池不存在</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeAlreadyActive</t>
+          <t>AttributePoolLocked</t>
         </is>
       </c>
       <c r="B238" s="0" t="inlineStr">
         <is>
-          <t>已经是当前方案</t>
+          <t>该属性池尚未解锁</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="0" t="inlineStr">
         <is>
-          <t>AttributeInBattle</t>
+          <t>AttributeDimensionNotFound</t>
         </is>
       </c>
       <c r="B239" s="0" t="inlineStr">
         <is>
-          <t>战斗中不能修改属性</t>
+          <t>属性维度不存在</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t>AttributeGoldNotEnough</t>
+          <t>AttributePointsNotEnough</t>
         </is>
       </c>
       <c r="B240" s="0" t="inlineStr">
         <is>
-          <t>金币不足</t>
+          <t>剩余点数不足</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t>AttributeNoAutoPlan</t>
+          <t>AttributePointsCannotDecrease</t>
         </is>
       </c>
       <c r="B241" s="0" t="inlineStr">
         <is>
-          <t>没有可用的自动加点方案</t>
+          <t>已分配的点数不能减少,请使用重置</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t>AttributeNothingToChange</t>
+          <t>AttributeDimensionCapExceeded</t>
         </is>
       </c>
       <c r="B242" s="0" t="inlineStr">
         <is>
-          <t>属性没有变化</t>
-        </is>
-      </c>
-    </row>
-    <row r="243"/>
+          <t>超过单项可分配上限</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="0" t="inlineStr">
+        <is>
+          <t>AttributeSchemeNotFound</t>
+        </is>
+      </c>
+      <c r="B243" s="0" t="inlineStr">
+        <is>
+          <t>加点方案不存在</t>
+        </is>
+      </c>
+    </row>
     <row r="244">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t>//pet_error base=26000 width=1000</t>
+          <t>AttributeSchemeLimitReached</t>
+        </is>
+      </c>
+      <c r="B244" s="0" t="inlineStr">
+        <is>
+          <t>加点方案数量已达上限</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t>PetNotFound</t>
+          <t>AttributeSchemeSwitchCooldown</t>
         </is>
       </c>
       <c r="B245" s="0" t="inlineStr">
         <is>
-          <t>宝宝不存在</t>
+          <t>方案切换冷却中</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t>PetTableRowMissing</t>
+          <t>AttributeSchemeNameInvalid</t>
         </is>
       </c>
       <c r="B246" s="0" t="inlineStr">
         <is>
-          <t>宝宝数据已失效,请联系客服</t>
+          <t>方案名称不合法</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t>PetSlotFull</t>
+          <t>AttributeSchemeAlreadyActive</t>
         </is>
       </c>
       <c r="B247" s="0" t="inlineStr">
         <is>
-          <t>可携带的宝宝数量已达上限</t>
+          <t>已经是当前方案</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t>PetOwnerLevelNotEnough</t>
+          <t>AttributeInBattle</t>
         </is>
       </c>
       <c r="B248" s="0" t="inlineStr">
         <is>
-          <t>主人等级不足,还不能携带这只宝宝</t>
+          <t>战斗中不能修改属性</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t>PetAlreadyActive</t>
+          <t>AttributeGoldNotEnough</t>
         </is>
       </c>
       <c r="B249" s="0" t="inlineStr">
         <is>
-          <t>这只宝宝已经在出战中</t>
+          <t>金币不足</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t>PetNotActive</t>
+          <t>AttributeNoAutoPlan</t>
         </is>
       </c>
       <c r="B250" s="0" t="inlineStr">
         <is>
-          <t>当前没有出战的宝宝</t>
+          <t>没有可用的自动加点方案</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t>PetSummonCooldown</t>
+          <t>AttributeNothingToChange</t>
         </is>
       </c>
       <c r="B251" s="0" t="inlineStr">
         <is>
-          <t>操作太频繁,请稍后再试</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="0" t="inlineStr">
-        <is>
-          <t>PetNameInvalid</t>
-        </is>
-      </c>
-      <c r="B252" s="0" t="inlineStr">
-        <is>
-          <t>宝宝名称不合法</t>
-        </is>
-      </c>
-    </row>
+          <t>属性没有变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="252"/>
     <row r="253">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t>PetInBattle</t>
-        </is>
-      </c>
-      <c r="B253" s="0" t="inlineStr">
-        <is>
-          <t>战斗中不能操作宝宝</t>
+          <t>//pet_error base=26000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t>PetPointsNotEnough</t>
+          <t>PetNotFound</t>
         </is>
       </c>
       <c r="B254" s="0" t="inlineStr">
         <is>
-          <t>宝宝剩余点数不足</t>
+          <t>宝宝不存在</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t>PetPointsCannotDecrease</t>
+          <t>PetTableRowMissing</t>
         </is>
       </c>
       <c r="B255" s="0" t="inlineStr">
         <is>
-          <t>已分配的点数不能减少,请使用洗点</t>
+          <t>宝宝数据已失效,请联系客服</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="0" t="inlineStr">
         <is>
-          <t>PetDimensionCapExceeded</t>
+          <t>PetSlotFull</t>
         </is>
       </c>
       <c r="B256" s="0" t="inlineStr">
         <is>
-          <t>超过单项可分配上限</t>
+          <t>可携带的宝宝数量已达上限</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t>PetDimensionNotFound</t>
+          <t>PetOwnerLevelNotEnough</t>
         </is>
       </c>
       <c r="B257" s="0" t="inlineStr">
         <is>
-          <t>宝宝属性维度不存在</t>
+          <t>主人等级不足,还不能携带这只宝宝</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t>PetGoldNotEnough</t>
+          <t>PetAlreadyActive</t>
         </is>
       </c>
       <c r="B258" s="0" t="inlineStr">
         <is>
-          <t>金币不足</t>
+          <t>这只宝宝已经在出战中</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="0" t="inlineStr">
         <is>
-          <t>PetNoAutoPlan</t>
+          <t>PetNotActive</t>
         </is>
       </c>
       <c r="B259" s="0" t="inlineStr">
         <is>
-          <t>没有可用的自动加点方案</t>
+          <t>当前没有出战的宝宝</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t>PetNothingToChange</t>
+          <t>PetSummonCooldown</t>
         </is>
       </c>
       <c r="B260" s="0" t="inlineStr">
         <is>
-          <t>宝宝属性没有变化</t>
+          <t>操作太频繁,请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="0" t="inlineStr">
         <is>
+          <t>PetNameInvalid</t>
+        </is>
+      </c>
+      <c r="B261" s="0" t="inlineStr">
+        <is>
+          <t>宝宝名称不合法</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="0" t="inlineStr">
+        <is>
+          <t>PetInBattle</t>
+        </is>
+      </c>
+      <c r="B262" s="0" t="inlineStr">
+        <is>
+          <t>战斗中不能操作宝宝</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="0" t="inlineStr">
+        <is>
+          <t>PetPointsNotEnough</t>
+        </is>
+      </c>
+      <c r="B263" s="0" t="inlineStr">
+        <is>
+          <t>宝宝剩余点数不足</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="0" t="inlineStr">
+        <is>
+          <t>PetPointsCannotDecrease</t>
+        </is>
+      </c>
+      <c r="B264" s="0" t="inlineStr">
+        <is>
+          <t>已分配的点数不能减少,请使用洗点</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="0" t="inlineStr">
+        <is>
+          <t>PetDimensionCapExceeded</t>
+        </is>
+      </c>
+      <c r="B265" s="0" t="inlineStr">
+        <is>
+          <t>超过单项可分配上限</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="0" t="inlineStr">
+        <is>
+          <t>PetDimensionNotFound</t>
+        </is>
+      </c>
+      <c r="B266" s="0" t="inlineStr">
+        <is>
+          <t>宝宝属性维度不存在</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="0" t="inlineStr">
+        <is>
+          <t>PetGoldNotEnough</t>
+        </is>
+      </c>
+      <c r="B267" s="0" t="inlineStr">
+        <is>
+          <t>金币不足</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="0" t="inlineStr">
+        <is>
+          <t>PetNoAutoPlan</t>
+        </is>
+      </c>
+      <c r="B268" s="0" t="inlineStr">
+        <is>
+          <t>没有可用的自动加点方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="0" t="inlineStr">
+        <is>
+          <t>PetNothingToChange</t>
+        </is>
+      </c>
+      <c r="B269" s="0" t="inlineStr">
+        <is>
+          <t>宝宝属性没有变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="0" t="inlineStr">
+        <is>
           <t>PetIdGenerateFailed</t>
         </is>
       </c>
-      <c r="B261" s="0" t="inlineStr">
+      <c r="B270" s="0" t="inlineStr">
         <is>
           <t>宝宝创建失败,请稍后再试</t>
         </is>
       </c>
-      <c r="C261" s="0" t="n">
+      <c r="C270" s="0" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP：每小时保存全部进度 2026-09-18 04:56:21 -04:00
</commit_message>
<xml_diff>
--- a/data/tip/Tip.xlsx
+++ b/data/tip/Tip.xlsx
@@ -1020,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C270"/>
+  <dimension ref="A1:C285"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="8" customWidth="1" style="2" min="3" max="3"/>
@@ -1953,206 +1953,210 @@
     <row r="96">
       <c r="A96" s="0" t="inlineStr">
         <is>
-          <t>//team_error base=4000 width=1000</t>
-        </is>
-      </c>
+          <t>ZoneTravelTargetZoneNotFound</t>
+        </is>
+      </c>
+      <c r="B96" s="0" t="inlineStr">
+        <is>
+          <t>目标区服不存在</t>
+        </is>
+      </c>
+      <c r="C96" s="0" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="0" t="inlineStr">
         <is>
-          <t>TeamNotInApplicants</t>
+          <t>ZoneTravelInBattle</t>
         </is>
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
-        </is>
-      </c>
+          <t>战斗中不能传送</t>
+        </is>
+      </c>
+      <c r="C97" s="0" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="0" t="inlineStr">
         <is>
-          <t>TeamPlayerId</t>
+          <t>ZoneTravelInTeam</t>
         </is>
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>玩家 ID 无效</t>
-        </is>
-      </c>
+          <t>组队中不能传送</t>
+        </is>
+      </c>
+      <c r="C98" s="0" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="0" t="inlineStr">
         <is>
-          <t>TeamMembersFull</t>
+          <t>ZoneTravelTargetBusy</t>
         </is>
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>队伍人数已满</t>
-        </is>
-      </c>
+          <t>目标区服繁忙,请稍后再试</t>
+        </is>
+      </c>
+      <c r="C99" s="0" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberInTeam</t>
-        </is>
-      </c>
-      <c r="B100" s="0" t="inlineStr">
-        <is>
-          <t>对方已经在队伍中</t>
+          <t>//team_error base=4000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberNotInTeam</t>
+          <t>TeamNotInApplicants</t>
         </is>
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>对方不在你的队伍中</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="0" t="inlineStr">
         <is>
-          <t>TeamKickSelf</t>
+          <t>TeamPlayerId</t>
         </is>
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t>不能把自己踢出队伍</t>
+          <t>玩家 ID 无效</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="0" t="inlineStr">
         <is>
-          <t>TeamKickNotLeader</t>
+          <t>TeamMembersFull</t>
         </is>
       </c>
       <c r="B103" s="0" t="inlineStr">
         <is>
-          <t>只有队长可以踢人</t>
+          <t>队伍人数已满</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="0" t="inlineStr">
         <is>
-          <t>TeamAppointSelf</t>
+          <t>TeamMemberInTeam</t>
         </is>
       </c>
       <c r="B104" s="0" t="inlineStr">
         <is>
-          <t>你已经是队长了</t>
+          <t>对方已经在队伍中</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="0" t="inlineStr">
         <is>
-          <t>TeamAppointLeaderNotLeader</t>
+          <t>TeamMemberNotInTeam</t>
         </is>
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t>只有队长可以转让队长</t>
+          <t>对方不在你的队伍中</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="0" t="inlineStr">
         <is>
-          <t>TeamFull</t>
+          <t>TeamKickSelf</t>
         </is>
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
+          <t>不能把自己踢出队伍</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="0" t="inlineStr">
         <is>
-          <t>TeamInApplicantList</t>
+          <t>TeamKickNotLeader</t>
         </is>
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
+          <t>只有队长可以踢人</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="0" t="inlineStr">
         <is>
-          <t>TeamNotInApplicantList</t>
+          <t>TeamAppointSelf</t>
         </is>
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t>该申请已失效</t>
+          <t>你已经是队长了</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="0" t="inlineStr">
         <is>
-          <t>TeamListMaxSize</t>
+          <t>TeamAppointLeaderNotLeader</t>
         </is>
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
+          <t>只有队长可以转让队长</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="0" t="inlineStr">
         <is>
-          <t>TeamHasNotTeamId</t>
+          <t>TeamFull</t>
         </is>
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t>你还没有队伍</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="0" t="inlineStr">
         <is>
-          <t>TeamDismissNotLeader</t>
+          <t>TeamInApplicantList</t>
         </is>
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t>只有队长可以解散队伍</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberListFull</t>
+          <t>TeamNotInApplicantList</t>
         </is>
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
+          <t>该申请已失效</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="0" t="inlineStr">
         <is>
-          <t>TeamCreateTeamMaxMemberSize</t>
+          <t>TeamListMaxSize</t>
         </is>
       </c>
       <c r="B113" s="0" t="inlineStr">
@@ -2164,220 +2168,233 @@
     <row r="114">
       <c r="A114" s="0" t="inlineStr">
         <is>
-          <t>TeamPlayerNotFound</t>
+          <t>TeamHasNotTeamId</t>
         </is>
       </c>
       <c r="B114" s="0" t="inlineStr">
         <is>
-          <t>找不到该玩家</t>
+          <t>你还没有队伍</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="0" t="inlineStr">
         <is>
-          <t>TeamNotLeader</t>
+          <t>TeamDismissNotLeader</t>
         </is>
       </c>
       <c r="B115" s="0" t="inlineStr">
         <is>
-          <t>只有队长可以执行此操作</t>
+          <t>只有队长可以解散队伍</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="0" t="inlineStr">
         <is>
-          <t>TeamHomeZoneUnknown</t>
+          <t>TeamMemberListFull</t>
         </is>
       </c>
       <c r="B116" s="0" t="inlineStr">
         <is>
-          <t>角色区服信息异常，请重新登录</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="0" t="inlineStr">
         <is>
-          <t>TeamCrossZoneDenied</t>
+          <t>TeamCreateTeamMaxMemberSize</t>
         </is>
       </c>
       <c r="B117" s="0" t="inlineStr">
         <is>
-          <t>不能与其他区服的玩家组队</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="0" t="inlineStr">
         <is>
-          <t>TeamInviteNotFound</t>
+          <t>TeamPlayerNotFound</t>
         </is>
       </c>
       <c r="B118" s="0" t="inlineStr">
         <is>
-          <t>邀请已失效</t>
+          <t>找不到该玩家</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="0" t="inlineStr">
         <is>
-          <t>TeamInviteLimit</t>
+          <t>TeamNotLeader</t>
         </is>
       </c>
       <c r="B119" s="0" t="inlineStr">
         <is>
-          <t>对方待处理的邀请过多，请稍后再试</t>
+          <t>只有队长可以执行此操作</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="0" t="inlineStr">
         <is>
-          <t>TeamInMatch</t>
+          <t>TeamHomeZoneUnknown</t>
         </is>
       </c>
       <c r="B120" s="0" t="inlineStr">
         <is>
-          <t>队伍正在进入战斗，请稍候</t>
+          <t>角色区服信息异常，请重新登录</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberOffline</t>
+          <t>TeamCrossZoneDenied</t>
         </is>
       </c>
       <c r="B121" s="0" t="inlineStr">
         <is>
-          <t>有队员不在线</t>
+          <t>不能与其他区服的玩家组队</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberInBattle</t>
+          <t>TeamInviteNotFound</t>
         </is>
       </c>
       <c r="B122" s="0" t="inlineStr">
         <is>
-          <t>有队员正在战斗中</t>
+          <t>邀请已失效</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberNotReady</t>
+          <t>TeamInviteLimit</t>
         </is>
       </c>
       <c r="B123" s="0" t="inlineStr">
         <is>
-          <t>有队员暂时无法开战</t>
+          <t>对方待处理的邀请过多，请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="0" t="inlineStr">
         <is>
-          <t>TeamDungeonNotOpen</t>
+          <t>TeamInMatch</t>
         </is>
       </c>
       <c r="B124" s="0" t="inlineStr">
         <is>
-          <t>该副本未开放组队</t>
+          <t>队伍正在进入战斗，请稍候</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="0" t="inlineStr">
         <is>
-          <t>TeamSizeExceeded</t>
+          <t>TeamMemberOffline</t>
         </is>
       </c>
       <c r="B125" s="0" t="inlineStr">
         <is>
-          <t>队伍人数超过该副本上限</t>
+          <t>有队员不在线</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="0" t="inlineStr">
         <is>
-          <t>TeamStateChanged</t>
+          <t>TeamMemberInBattle</t>
         </is>
       </c>
       <c r="B126" s="0" t="inlineStr">
         <is>
-          <t>队伍状态已变化，请重试</t>
+          <t>有队员正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="0" t="inlineStr">
         <is>
-          <t>TeamInternal</t>
+          <t>TeamMemberNotReady</t>
         </is>
       </c>
       <c r="B127" s="0" t="inlineStr">
         <is>
-          <t>服务器繁忙，请稍后再试</t>
-        </is>
-      </c>
-      <c r="C127" s="0" t="n">
-        <v>1</v>
+          <t>有队员暂时无法开战</t>
+        </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="0" t="inlineStr">
         <is>
-          <t>//mission_error base=5000 width=1000</t>
+          <t>TeamDungeonNotOpen</t>
+        </is>
+      </c>
+      <c r="B128" s="0" t="inlineStr">
+        <is>
+          <t>该副本未开放组队</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="0" t="inlineStr">
         <is>
-          <t>MissionTypeAlreadyExists</t>
-        </is>
-      </c>
-      <c r="B129" s="0" t="inlineStr"/>
+          <t>TeamSizeExceeded</t>
+        </is>
+      </c>
+      <c r="B129" s="0" t="inlineStr">
+        <is>
+          <t>队伍人数超过该副本上限</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="0" t="inlineStr">
         <is>
-          <t>MissionAlreadyCompleted</t>
-        </is>
-      </c>
-      <c r="B130" s="0" t="inlineStr"/>
+          <t>TeamStateChanged</t>
+        </is>
+      </c>
+      <c r="B130" s="0" t="inlineStr">
+        <is>
+          <t>队伍状态已变化，请重试</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="0" t="inlineStr">
         <is>
-          <t>MissionIdNotInRewardList</t>
-        </is>
-      </c>
-      <c r="B131" s="0" t="inlineStr"/>
+          <t>TeamInternal</t>
+        </is>
+      </c>
+      <c r="B131" s="0" t="inlineStr">
+        <is>
+          <t>服务器繁忙，请稍后再试</t>
+        </is>
+      </c>
+      <c r="C131" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="0" t="inlineStr">
         <is>
-          <t>PlayerMissionComponentNotFound</t>
-        </is>
-      </c>
-      <c r="B132" s="0" t="inlineStr"/>
-      <c r="C132" s="0" t="n">
-        <v>1</v>
+          <t>//mission_error base=5000 width=1000</t>
+        </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="0" t="inlineStr">
         <is>
-          <t>MissionIdRepeated</t>
+          <t>MissionTypeAlreadyExists</t>
         </is>
       </c>
       <c r="B133" s="0" t="inlineStr"/>
@@ -2385,7 +2402,7 @@
     <row r="134">
       <c r="A134" s="0" t="inlineStr">
         <is>
-          <t>ConditionIdOutOfRange</t>
+          <t>MissionAlreadyCompleted</t>
         </is>
       </c>
       <c r="B134" s="0" t="inlineStr"/>
@@ -2393,7 +2410,7 @@
     <row r="135">
       <c r="A135" s="0" t="inlineStr">
         <is>
-          <t>MissionNotInProgress</t>
+          <t>MissionIdNotInRewardList</t>
         </is>
       </c>
       <c r="B135" s="0" t="inlineStr"/>
@@ -2401,14 +2418,18 @@
     <row r="136">
       <c r="A136" s="0" t="inlineStr">
         <is>
-          <t>//bag_error base=6000 width=1000</t>
-        </is>
+          <t>PlayerMissionComponentNotFound</t>
+        </is>
+      </c>
+      <c r="B136" s="0" t="inlineStr"/>
+      <c r="C136" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="0" t="inlineStr">
         <is>
-          <t>BagDeleteItemFindGuid</t>
+          <t>MissionIdRepeated</t>
         </is>
       </c>
       <c r="B137" s="0" t="inlineStr"/>
@@ -2416,7 +2437,7 @@
     <row r="138">
       <c r="A138" s="0" t="inlineStr">
         <is>
-          <t>BagDeleteItemAlreadyHasGuid</t>
+          <t>ConditionIdOutOfRange</t>
         </is>
       </c>
       <c r="B138" s="0" t="inlineStr"/>
@@ -2424,26 +2445,22 @@
     <row r="139">
       <c r="A139" s="0" t="inlineStr">
         <is>
-          <t>BagAddItemHasNotBaseComponent</t>
+          <t>MissionNotInProgress</t>
         </is>
       </c>
       <c r="B139" s="0" t="inlineStr"/>
-      <c r="C139" s="0" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="140">
       <c r="A140" s="0" t="inlineStr">
         <is>
-          <t>BagAddItemInvalidGuid</t>
-        </is>
-      </c>
-      <c r="B140" s="0" t="inlineStr"/>
+          <t>//bag_error base=6000 width=1000</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="0" t="inlineStr">
         <is>
-          <t>BagAddItemInvalidParam</t>
+          <t>BagDeleteItemFindGuid</t>
         </is>
       </c>
       <c r="B141" s="0" t="inlineStr"/>
@@ -2451,7 +2468,7 @@
     <row r="142">
       <c r="A142" s="0" t="inlineStr">
         <is>
-          <t>BagAddItemBagFull</t>
+          <t>BagDeleteItemAlreadyHasGuid</t>
         </is>
       </c>
       <c r="B142" s="0" t="inlineStr"/>
@@ -2459,15 +2476,18 @@
     <row r="143">
       <c r="A143" s="0" t="inlineStr">
         <is>
-          <t>BagItemNotStacked</t>
+          <t>BagAddItemHasNotBaseComponent</t>
         </is>
       </c>
       <c r="B143" s="0" t="inlineStr"/>
+      <c r="C143" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="0" t="inlineStr">
         <is>
-          <t>BagInsufficientItems</t>
+          <t>BagAddItemInvalidGuid</t>
         </is>
       </c>
       <c r="B144" s="0" t="inlineStr"/>
@@ -2475,7 +2495,7 @@
     <row r="145">
       <c r="A145" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemPos</t>
+          <t>BagAddItemInvalidParam</t>
         </is>
       </c>
       <c r="B145" s="0" t="inlineStr"/>
@@ -2483,7 +2503,7 @@
     <row r="146">
       <c r="A146" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemConfig</t>
+          <t>BagAddItemBagFull</t>
         </is>
       </c>
       <c r="B146" s="0" t="inlineStr"/>
@@ -2491,7 +2511,7 @@
     <row r="147">
       <c r="A147" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemGuid</t>
+          <t>BagItemNotStacked</t>
         </is>
       </c>
       <c r="B147" s="0" t="inlineStr"/>
@@ -2499,7 +2519,7 @@
     <row r="148">
       <c r="A148" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemFindItem</t>
+          <t>BagInsufficientItems</t>
         </is>
       </c>
       <c r="B148" s="0" t="inlineStr"/>
@@ -2507,7 +2527,7 @@
     <row r="149">
       <c r="A149" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemSize</t>
+          <t>BagDelItemPos</t>
         </is>
       </c>
       <c r="B149" s="0" t="inlineStr"/>
@@ -2515,7 +2535,7 @@
     <row r="150">
       <c r="A150" s="0" t="inlineStr">
         <is>
-          <t>BagItemDeletionSizeMismatch</t>
+          <t>BagDelItemConfig</t>
         </is>
       </c>
       <c r="B150" s="0" t="inlineStr"/>
@@ -2523,7 +2543,7 @@
     <row r="151">
       <c r="A151" s="0" t="inlineStr">
         <is>
-          <t>BagInsufficientBagSpace</t>
+          <t>BagDelItemGuid</t>
         </is>
       </c>
       <c r="B151" s="0" t="inlineStr"/>
@@ -2531,1321 +2551,1477 @@
     <row r="152">
       <c r="A152" s="0" t="inlineStr">
         <is>
-          <t>//skill_error base=7000 width=1000</t>
-        </is>
-      </c>
+          <t>BagDelItemFindItem</t>
+        </is>
+      </c>
+      <c r="B152" s="0" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="0" t="inlineStr">
         <is>
-          <t>SkillUnInterruptible</t>
-        </is>
-      </c>
-      <c r="B153" s="0" t="inlineStr">
-        <is>
-          <t>技能不能被打断</t>
-        </is>
-      </c>
+          <t>BagDelItemSize</t>
+        </is>
+      </c>
+      <c r="B153" s="0" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="0" t="inlineStr">
         <is>
-          <t>SkillInvalidTargetId</t>
-        </is>
-      </c>
-      <c r="B154" s="0" t="inlineStr">
-        <is>
-          <t>目标id错误</t>
-        </is>
-      </c>
+          <t>BagItemDeletionSizeMismatch</t>
+        </is>
+      </c>
+      <c r="B154" s="0" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="0" t="inlineStr">
         <is>
-          <t>SkillInvalidTarget</t>
-        </is>
-      </c>
-      <c r="B155" s="0" t="inlineStr">
-        <is>
-          <t>未找到释放目标</t>
-        </is>
-      </c>
+          <t>BagInsufficientBagSpace</t>
+        </is>
+      </c>
+      <c r="B155" s="0" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="0" t="inlineStr">
         <is>
-          <t>SkillCooldownNotReady</t>
-        </is>
-      </c>
-      <c r="B156" s="0" t="inlineStr">
-        <is>
-          <t>技能冷却尚未完成，无法使用技能</t>
+          <t>//skill_error base=7000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="0" t="inlineStr">
         <is>
-          <t>SkillCannotBeCastInCurrentState</t>
+          <t>SkillUnInterruptible</t>
         </is>
       </c>
       <c r="B157" s="0" t="inlineStr">
         <is>
-          <t>当前状态不能释放该技能</t>
+          <t>技能不能被打断</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="0" t="inlineStr">
         <is>
-          <t>SkillCannotBeCastSilenceRestriction</t>
+          <t>SkillInvalidTargetId</t>
         </is>
       </c>
       <c r="B158" s="0" t="inlineStr">
         <is>
-          <t>当前沉默状态不能释放该技能</t>
+          <t>目标id错误</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="0" t="inlineStr">
         <is>
-          <t>SkillCannotBeCastStunRestriction</t>
+          <t>SkillInvalidTarget</t>
         </is>
       </c>
       <c r="B159" s="0" t="inlineStr">
         <is>
-          <t>当前眩晕状态不能释放该技能</t>
+          <t>未找到释放目标</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="0" t="inlineStr">
         <is>
-          <t>//buff_error base=8000 width=1000</t>
+          <t>SkillCooldownNotReady</t>
+        </is>
+      </c>
+      <c r="B160" s="0" t="inlineStr">
+        <is>
+          <t>技能冷却尚未完成，无法使用技能</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="0" t="inlineStr">
         <is>
-          <t>BuffMaxBuffStack</t>
+          <t>SkillCannotBeCastInCurrentState</t>
         </is>
       </c>
       <c r="B161" s="0" t="inlineStr">
         <is>
-          <t>buff层数已经最大</t>
+          <t>当前状态不能释放该技能</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="0" t="inlineStr">
         <is>
-          <t>BuffTargetImmuneToBuff</t>
+          <t>SkillCannotBeCastSilenceRestriction</t>
         </is>
       </c>
       <c r="B162" s="0" t="inlineStr">
         <is>
-          <t>目标免疫buff</t>
+          <t>当前沉默状态不能释放该技能</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="0" t="inlineStr">
         <is>
-          <t>//entity_error base=9000 width=1000</t>
+          <t>SkillCannotBeCastStunRestriction</t>
+        </is>
+      </c>
+      <c r="B163" s="0" t="inlineStr">
+        <is>
+          <t>当前眩晕状态不能释放该技能</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="0" t="inlineStr">
         <is>
-          <t>EntityTransformNotFound</t>
-        </is>
-      </c>
-      <c r="B164" s="0" t="inlineStr">
-        <is>
-          <t>未找到实体的Transfor组件</t>
-        </is>
-      </c>
-      <c r="C164" s="0" t="n">
-        <v>1</v>
+          <t>//buff_error base=8000 width=1000</t>
+        </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="0" t="inlineStr">
         <is>
-          <t>//actor_action_error base=10000 width=1000</t>
+          <t>BuffMaxBuffStack</t>
+        </is>
+      </c>
+      <c r="B165" s="0" t="inlineStr">
+        <is>
+          <t>buff层数已经最大</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="0" t="inlineStr">
         <is>
-          <t>ActorActionStateActionCannotBePerformedWhileInTeamFollowMode</t>
+          <t>BuffTargetImmuneToBuff</t>
         </is>
       </c>
       <c r="B166" s="0" t="inlineStr">
         <is>
-          <t>正在组队跟随中</t>
+          <t>目标免疫buff</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="0" t="inlineStr">
         <is>
-          <t>//mount_error base=11000 width=1000</t>
+          <t>//entity_error base=9000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="0" t="inlineStr">
         <is>
-          <t>MountNotMounted</t>
+          <t>EntityTransformNotFound</t>
         </is>
       </c>
       <c r="B168" s="0" t="inlineStr">
         <is>
-          <t>当前不在坐骑上</t>
-        </is>
+          <t>未找到实体的Transfor组件</t>
+        </is>
+      </c>
+      <c r="C168" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="0" t="inlineStr">
         <is>
-          <t>//reward_error base=12000 width=1000</t>
+          <t>//actor_action_error base=10000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="0" t="inlineStr">
         <is>
-          <t>RewardAlreadyClaimed</t>
+          <t>ActorActionStateActionCannotBePerformedWhileInTeamFollowMode</t>
         </is>
       </c>
       <c r="B170" s="0" t="inlineStr">
         <is>
-          <t>该奖励已经领取过了</t>
+          <t>正在组队跟随中</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="0" t="inlineStr">
         <is>
-          <t>//cross_server_error base=13000 width=1000</t>
+          <t>//mount_error base=11000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="0" t="inlineStr">
         <is>
-          <t>SceneTransferInProgress</t>
-        </is>
-      </c>
-      <c r="B172" s="0" t="inlineStr"/>
+          <t>MountNotMounted</t>
+        </is>
+      </c>
+      <c r="B172" s="0" t="inlineStr">
+        <is>
+          <t>当前不在坐骑上</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="0" t="inlineStr">
         <is>
-          <t>//guild_error base=14000 width=1000</t>
+          <t>//reward_error base=12000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="0" t="inlineStr">
         <is>
-          <t>GuildAlreadyInGuild</t>
+          <t>RewardAlreadyClaimed</t>
         </is>
       </c>
       <c r="B174" s="0" t="inlineStr">
         <is>
-          <t>已加入公会</t>
+          <t>该奖励已经领取过了</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="0" t="inlineStr">
         <is>
-          <t>GuildNotFound</t>
-        </is>
-      </c>
-      <c r="B175" s="0" t="inlineStr">
-        <is>
-          <t>公会不存在</t>
+          <t>//cross_server_error base=13000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="0" t="inlineStr">
         <is>
-          <t>GuildNotInGuild</t>
-        </is>
-      </c>
-      <c r="B176" s="0" t="inlineStr">
-        <is>
-          <t>尚未加入公会</t>
-        </is>
-      </c>
+          <t>SceneTransferInProgress</t>
+        </is>
+      </c>
+      <c r="B176" s="0" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t>GuildFull</t>
-        </is>
-      </c>
-      <c r="B177" s="0" t="inlineStr">
-        <is>
-          <t>公会人数已满</t>
+          <t>//guild_error base=14000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t>GuildLeaderCantLeave</t>
+          <t>GuildAlreadyInGuild</t>
         </is>
       </c>
       <c r="B178" s="0" t="inlineStr">
         <is>
-          <t>会长不能退出公会</t>
+          <t>已加入公会</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t>GuildNotLeader</t>
+          <t>GuildNotFound</t>
         </is>
       </c>
       <c r="B179" s="0" t="inlineStr">
         <is>
-          <t>只有会长可以执行该操作</t>
+          <t>公会不存在</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t>GuildNoPermission</t>
+          <t>GuildNotInGuild</t>
         </is>
       </c>
       <c r="B180" s="0" t="inlineStr">
         <is>
-          <t>权限不足</t>
+          <t>尚未加入公会</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t>GuildNotRanked</t>
+          <t>GuildFull</t>
         </is>
       </c>
       <c r="B181" s="0" t="inlineStr">
         <is>
-          <t>暂未上榜</t>
+          <t>公会人数已满</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t>GuildIdGenUnavailable</t>
+          <t>GuildLeaderCantLeave</t>
         </is>
       </c>
       <c r="B182" s="0" t="inlineStr">
         <is>
-          <t>服务繁忙，请稍后重试</t>
-        </is>
-      </c>
-      <c r="C182" s="0" t="n">
-        <v>1</v>
+          <t>会长不能退出公会</t>
+        </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t>GuildNameInvalid</t>
+          <t>GuildNotLeader</t>
         </is>
       </c>
       <c r="B183" s="0" t="inlineStr">
         <is>
-          <t>公会名称无效（1-24 个字，不能包含控制字符）</t>
+          <t>只有会长可以执行该操作</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t>GuildNameTaken</t>
+          <t>GuildNoPermission</t>
         </is>
       </c>
       <c r="B184" s="0" t="inlineStr">
         <is>
-          <t>公会名称已被使用</t>
+          <t>权限不足</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t>GuildAnnouncementTooLong</t>
+          <t>GuildNotRanked</t>
         </is>
       </c>
       <c r="B185" s="0" t="inlineStr">
         <is>
-          <t>公会公告过长</t>
+          <t>暂未上榜</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="0" t="inlineStr">
         <is>
+          <t>GuildIdGenUnavailable</t>
+        </is>
+      </c>
+      <c r="B186" s="0" t="inlineStr">
+        <is>
+          <t>服务繁忙，请稍后重试</t>
+        </is>
+      </c>
+      <c r="C186" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="0" t="inlineStr">
+        <is>
+          <t>GuildNameInvalid</t>
+        </is>
+      </c>
+      <c r="B187" s="0" t="inlineStr">
+        <is>
+          <t>公会名称无效（1-24 个字，不能包含控制字符）</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="0" t="inlineStr">
+        <is>
+          <t>GuildNameTaken</t>
+        </is>
+      </c>
+      <c r="B188" s="0" t="inlineStr">
+        <is>
+          <t>公会名称已被使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="0" t="inlineStr">
+        <is>
+          <t>GuildAnnouncementTooLong</t>
+        </is>
+      </c>
+      <c r="B189" s="0" t="inlineStr">
+        <is>
+          <t>公会公告过长</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="0" t="inlineStr">
+        <is>
           <t>GuildHomeZoneUnknown</t>
         </is>
       </c>
-      <c r="B186" s="0" t="inlineStr">
+      <c r="B190" s="0" t="inlineStr">
         <is>
           <t>角色归属区服未确认，暂时无法使用公会</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="0" t="inlineStr">
         <is>
           <t>GuildZoneMerging</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr">
+      <c r="B191" s="0" t="inlineStr">
         <is>
           <t>区服合并维护中，帮会操作暂停，请稍后再试</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="0" t="inlineStr">
         <is>
           <t>GuildTargetNotMember</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr">
+      <c r="B192" s="0" t="inlineStr">
         <is>
           <t>对方已不在本帮会</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="0" t="inlineStr">
         <is>
           <t>GuildCannotTargetSelf</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr">
+      <c r="B193" s="0" t="inlineStr">
         <is>
           <t>不能对自己执行此操作</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="0" t="inlineStr">
         <is>
           <t>GuildRankTooLow</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
+      <c r="B194" s="0" t="inlineStr">
         <is>
           <t>帮会职位不足，无法执行此操作</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
+    <row r="195">
+      <c r="A195" s="0" t="inlineStr">
         <is>
           <t>GuildOfficerLimit</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr">
+      <c r="B195" s="0" t="inlineStr">
         <is>
           <t>长老人数已达当前帮会等级上限</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>GuildApplicationNotFound</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>入帮申请不存在或已失效</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>GuildApplicationLimit</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>同时进行中的入帮申请已达上限</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>GuildApplicationQueueFull</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>该帮会待审申请已满，请稍后再试</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>GuildBusyRetry</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>帮会操作繁忙，请稍后重试</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t>//friend_error base=15000 width=1000</t>
+          <t>GuildApplicationNotFound</t>
+        </is>
+      </c>
+      <c r="B196" s="0" t="inlineStr">
+        <is>
+          <t>入帮申请不存在或已失效</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t>FriendCannotAddSelf</t>
+          <t>GuildApplicationLimit</t>
         </is>
       </c>
       <c r="B197" s="0" t="inlineStr">
         <is>
-          <t>不能添加自己为好友</t>
+          <t>同时进行中的入帮申请已达上限</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t>FriendAlreadyFriends</t>
+          <t>GuildApplicationQueueFull</t>
         </is>
       </c>
       <c r="B198" s="0" t="inlineStr">
         <is>
-          <t>你们已经是好友了</t>
+          <t>该帮会待审申请已满，请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t>FriendListFull</t>
+          <t>GuildBusyRetry</t>
         </is>
       </c>
       <c r="B199" s="0" t="inlineStr">
         <is>
-          <t>好友列表已满</t>
+          <t>帮会操作繁忙，请稍后重试</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t>FriendRequestAlreadySent</t>
-        </is>
-      </c>
-      <c r="B200" s="0" t="inlineStr">
-        <is>
-          <t>已发送过好友申请</t>
+          <t>//friend_error base=15000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t>FriendTargetListFull</t>
+          <t>FriendCannotAddSelf</t>
         </is>
       </c>
       <c r="B201" s="0" t="inlineStr">
         <is>
-          <t>对方好友列表已满</t>
+          <t>不能添加自己为好友</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t>FriendNoPendingRequest</t>
+          <t>FriendAlreadyFriends</t>
         </is>
       </c>
       <c r="B202" s="0" t="inlineStr">
         <is>
-          <t>没有待处理的好友申请</t>
+          <t>你们已经是好友了</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>FriendTooManyPending</t>
+          <t>FriendListFull</t>
         </is>
       </c>
       <c r="B203" s="0" t="inlineStr">
         <is>
-          <t>待处理的申请过多</t>
+          <t>好友列表已满</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t>//match_error base=16000 width=1000</t>
+          <t>FriendRequestAlreadySent</t>
+        </is>
+      </c>
+      <c r="B204" s="0" t="inlineStr">
+        <is>
+          <t>已发送过好友申请</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t>MatchInBattle</t>
+          <t>FriendTargetListFull</t>
         </is>
       </c>
       <c r="B205" s="0" t="inlineStr">
         <is>
-          <t>你正在战斗中</t>
+          <t>对方好友列表已满</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t>MatchAlreadyQueued</t>
+          <t>FriendNoPendingRequest</t>
         </is>
       </c>
       <c r="B206" s="0" t="inlineStr">
         <is>
-          <t>已在匹配队列中</t>
+          <t>没有待处理的好友申请</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t>MatchModeNotOpen</t>
+          <t>FriendTooManyPending</t>
         </is>
       </c>
       <c r="B207" s="0" t="inlineStr">
         <is>
-          <t>该匹配模式暂未开放</t>
+          <t>待处理的申请过多</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t>MatchTeamSizeNotConfigured</t>
-        </is>
-      </c>
-      <c r="B208" s="0" t="inlineStr">
-        <is>
-          <t>队伍人数未配置</t>
+          <t>//match_error base=16000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t>MatchInternal</t>
+          <t>MatchInBattle</t>
         </is>
       </c>
       <c r="B209" s="0" t="inlineStr">
         <is>
-          <t>服务繁忙，请稍后重试</t>
-        </is>
-      </c>
-      <c r="C209" s="0" t="n"/>
+          <t>你正在战斗中</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t>MatchTicketMismatch</t>
+          <t>MatchAlreadyQueued</t>
         </is>
       </c>
       <c r="B210" s="0" t="inlineStr">
         <is>
-          <t>匹配凭据不匹配</t>
+          <t>已在匹配队列中</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t>MatchCancelTooLate</t>
+          <t>MatchModeNotOpen</t>
         </is>
       </c>
       <c r="B211" s="0" t="inlineStr">
         <is>
-          <t>匹配已开始，无法取消</t>
+          <t>该匹配模式暂未开放</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeSelf</t>
+          <t>MatchTeamSizeNotConfigured</t>
         </is>
       </c>
       <c r="B212" s="0" t="inlineStr">
         <is>
-          <t>不能挑战自己</t>
+          <t>队伍人数未配置</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeTargetOffline</t>
+          <t>MatchInternal</t>
         </is>
       </c>
       <c r="B213" s="0" t="inlineStr">
         <is>
-          <t>对方不在线</t>
-        </is>
-      </c>
+          <t>服务繁忙，请稍后重试</t>
+        </is>
+      </c>
+      <c r="C213" s="0" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeTargetBusy</t>
+          <t>MatchTicketMismatch</t>
         </is>
       </c>
       <c r="B214" s="0" t="inlineStr">
         <is>
-          <t>对方正在战斗中</t>
+          <t>匹配凭据不匹配</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeSelfBusy</t>
+          <t>MatchCancelTooLate</t>
         </is>
       </c>
       <c r="B215" s="0" t="inlineStr">
         <is>
-          <t>你正在战斗中</t>
+          <t>匹配已开始，无法取消</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengePending</t>
+          <t>MatchChallengeSelf</t>
         </is>
       </c>
       <c r="B216" s="0" t="inlineStr">
         <is>
-          <t>已有待应答的挑战</t>
+          <t>不能挑战自己</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeExpired</t>
+          <t>MatchChallengeTargetOffline</t>
         </is>
       </c>
       <c r="B217" s="0" t="inlineStr">
         <is>
-          <t>挑战已过期</t>
+          <t>对方不在线</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeNotTarget</t>
+          <t>MatchChallengeTargetBusy</t>
         </is>
       </c>
       <c r="B218" s="0" t="inlineStr">
         <is>
-          <t>你不是该挑战的对象</t>
+          <t>对方正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateWhileQueued</t>
+          <t>MatchChallengeSelfBusy</t>
         </is>
       </c>
       <c r="B219" s="0" t="inlineStr">
         <is>
-          <t>匹配中无法观战</t>
+          <t>你正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateWhileInBattle</t>
+          <t>MatchChallengePending</t>
         </is>
       </c>
       <c r="B220" s="0" t="inlineStr">
         <is>
-          <t>战斗中无法观战</t>
+          <t>已有待应答的挑战</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t>MatchAlreadyWatching</t>
+          <t>MatchChallengeExpired</t>
         </is>
       </c>
       <c r="B221" s="0" t="inlineStr">
         <is>
-          <t>已在观战中</t>
+          <t>挑战已过期</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t>MatchNoWatchableBattle</t>
+          <t>MatchChallengeNotTarget</t>
         </is>
       </c>
       <c r="B222" s="0" t="inlineStr">
         <is>
-          <t>当前没有可观战的战斗</t>
+          <t>你不是该挑战的对象</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t>MatchBattleNotWatchable</t>
+          <t>MatchSpectateWhileQueued</t>
         </is>
       </c>
       <c r="B223" s="0" t="inlineStr">
         <is>
-          <t>该战斗无法观战</t>
+          <t>匹配中无法观战</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateOffline</t>
+          <t>MatchSpectateWhileInBattle</t>
         </is>
       </c>
       <c r="B224" s="0" t="inlineStr">
         <is>
-          <t>观战会话已断开</t>
+          <t>战斗中无法观战</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t>MatchNotInScene</t>
+          <t>MatchAlreadyWatching</t>
         </is>
       </c>
       <c r="B225" s="0" t="inlineStr">
         <is>
-          <t>请先进入场景</t>
+          <t>已在观战中</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t>// 以下号段为移植域预留，建组时把本行改成组头即可：</t>
+          <t>MatchNoWatchableBattle</t>
+        </is>
+      </c>
+      <c r="B226" s="0" t="inlineStr">
+        <is>
+          <t>当前没有可观战的战斗</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t>//   mail_error 17000 / chat_error 18000 / auction_error 19000</t>
+          <t>MatchBattleNotWatchable</t>
+        </is>
+      </c>
+      <c r="B227" s="0" t="inlineStr">
+        <is>
+          <t>该战斗无法观战</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t>//   rank_error 21000 / dialogue_error 22000 / battle_result_error 23000 / grant_error 24000</t>
-        </is>
-      </c>
-    </row>
-    <row r="229"/>
+          <t>MatchSpectateOffline</t>
+        </is>
+      </c>
+      <c r="B228" s="0" t="inlineStr">
+        <is>
+          <t>观战会话已断开</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="0" t="inlineStr">
+        <is>
+          <t>MatchNotInScene</t>
+        </is>
+      </c>
+      <c r="B229" s="0" t="inlineStr">
+        <is>
+          <t>请先进入场景</t>
+        </is>
+      </c>
+    </row>
     <row r="230">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t>//trade_error base=20000 width=1000</t>
+          <t>// 以下号段为移植域预留，建组时把本行改成组头即可：</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t>TradeListingNotFound</t>
-        </is>
-      </c>
-      <c r="B231" s="0" t="inlineStr">
-        <is>
-          <t>商品不存在或已下架</t>
+          <t>//   mail_error 17000 / chat_error 18000 / auction_error 19000</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t>TradeHomeZoneUnknown</t>
-        </is>
-      </c>
-      <c r="B232" s="0" t="inlineStr">
-        <is>
-          <t>角色归属区服未确认，暂时无法使用聚宝斋</t>
-        </is>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" s="0" t="inlineStr">
-        <is>
-          <t>TradeFavoriteLimitReached</t>
-        </is>
-      </c>
-      <c r="B233" s="0" t="inlineStr">
-        <is>
-          <t>收藏数量已达上限，请先取消部分收藏</t>
-        </is>
-      </c>
-    </row>
+          <t>//   rank_error 21000 / dialogue_error 22000 / battle_result_error 23000 / grant_error 24000</t>
+        </is>
+      </c>
+    </row>
+    <row r="233"/>
     <row r="234">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t>TradeFeatureDisabled</t>
-        </is>
-      </c>
-      <c r="B234" s="0" t="inlineStr">
-        <is>
-          <t>该功能尚未开放</t>
-        </is>
-      </c>
-    </row>
-    <row r="235"/>
+          <t>//trade_error base=20000 width=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="0" t="inlineStr">
+        <is>
+          <t>TradeListingNotFound</t>
+        </is>
+      </c>
+      <c r="B235" s="0" t="inlineStr">
+        <is>
+          <t>商品不存在或已下架</t>
+        </is>
+      </c>
+    </row>
     <row r="236">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t>//attribute_error base=25000 width=1000</t>
+          <t>TradeHomeZoneUnknown</t>
+        </is>
+      </c>
+      <c r="B236" s="0" t="inlineStr">
+        <is>
+          <t>角色归属区服未确认，暂时无法使用聚宝斋</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t>AttributePoolNotFound</t>
+          <t>TradeFavoriteLimitReached</t>
         </is>
       </c>
       <c r="B237" s="0" t="inlineStr">
         <is>
-          <t>属性池不存在</t>
+          <t>收藏数量已达上限，请先取消部分收藏</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t>AttributePoolLocked</t>
+          <t>TradeFeatureDisabled</t>
         </is>
       </c>
       <c r="B238" s="0" t="inlineStr">
         <is>
-          <t>该属性池尚未解锁</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" s="0" t="inlineStr">
-        <is>
-          <t>AttributeDimensionNotFound</t>
-        </is>
-      </c>
-      <c r="B239" s="0" t="inlineStr">
-        <is>
-          <t>属性维度不存在</t>
-        </is>
-      </c>
-    </row>
+          <t>该功能尚未开放</t>
+        </is>
+      </c>
+    </row>
+    <row r="239"/>
     <row r="240">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t>AttributePointsNotEnough</t>
-        </is>
-      </c>
-      <c r="B240" s="0" t="inlineStr">
-        <is>
-          <t>剩余点数不足</t>
+          <t>//attribute_error base=25000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t>AttributePointsCannotDecrease</t>
+          <t>AttributePoolNotFound</t>
         </is>
       </c>
       <c r="B241" s="0" t="inlineStr">
         <is>
-          <t>已分配的点数不能减少,请使用重置</t>
+          <t>属性池不存在</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t>AttributeDimensionCapExceeded</t>
+          <t>AttributePoolLocked</t>
         </is>
       </c>
       <c r="B242" s="0" t="inlineStr">
         <is>
-          <t>超过单项可分配上限</t>
+          <t>该属性池尚未解锁</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeNotFound</t>
+          <t>AttributeDimensionNotFound</t>
         </is>
       </c>
       <c r="B243" s="0" t="inlineStr">
         <is>
-          <t>加点方案不存在</t>
+          <t>属性维度不存在</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeLimitReached</t>
+          <t>AttributePointsNotEnough</t>
         </is>
       </c>
       <c r="B244" s="0" t="inlineStr">
         <is>
-          <t>加点方案数量已达上限</t>
+          <t>剩余点数不足</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeSwitchCooldown</t>
+          <t>AttributePointsCannotDecrease</t>
         </is>
       </c>
       <c r="B245" s="0" t="inlineStr">
         <is>
-          <t>方案切换冷却中</t>
+          <t>已分配的点数不能减少,请使用重置</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeNameInvalid</t>
+          <t>AttributeDimensionCapExceeded</t>
         </is>
       </c>
       <c r="B246" s="0" t="inlineStr">
         <is>
-          <t>方案名称不合法</t>
+          <t>超过单项可分配上限</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeAlreadyActive</t>
+          <t>AttributeSchemeNotFound</t>
         </is>
       </c>
       <c r="B247" s="0" t="inlineStr">
         <is>
-          <t>已经是当前方案</t>
+          <t>加点方案不存在</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t>AttributeInBattle</t>
+          <t>AttributeSchemeLimitReached</t>
         </is>
       </c>
       <c r="B248" s="0" t="inlineStr">
         <is>
-          <t>战斗中不能修改属性</t>
+          <t>加点方案数量已达上限</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t>AttributeGoldNotEnough</t>
+          <t>AttributeSchemeSwitchCooldown</t>
         </is>
       </c>
       <c r="B249" s="0" t="inlineStr">
         <is>
-          <t>金币不足</t>
+          <t>方案切换冷却中</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t>AttributeNoAutoPlan</t>
+          <t>AttributeSchemeNameInvalid</t>
         </is>
       </c>
       <c r="B250" s="0" t="inlineStr">
         <is>
-          <t>没有可用的自动加点方案</t>
+          <t>方案名称不合法</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t>AttributeNothingToChange</t>
+          <t>AttributeSchemeAlreadyActive</t>
         </is>
       </c>
       <c r="B251" s="0" t="inlineStr">
         <is>
-          <t>属性没有变化</t>
-        </is>
-      </c>
-    </row>
-    <row r="252"/>
+          <t>已经是当前方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="0" t="inlineStr">
+        <is>
+          <t>AttributeInBattle</t>
+        </is>
+      </c>
+      <c r="B252" s="0" t="inlineStr">
+        <is>
+          <t>战斗中不能修改属性</t>
+        </is>
+      </c>
+    </row>
     <row r="253">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t>//pet_error base=26000 width=1000</t>
+          <t>AttributeGoldNotEnough</t>
+        </is>
+      </c>
+      <c r="B253" s="0" t="inlineStr">
+        <is>
+          <t>金币不足</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t>PetNotFound</t>
+          <t>AttributeNoAutoPlan</t>
         </is>
       </c>
       <c r="B254" s="0" t="inlineStr">
         <is>
-          <t>宝宝不存在</t>
+          <t>没有可用的自动加点方案</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t>PetTableRowMissing</t>
+          <t>AttributeNothingToChange</t>
         </is>
       </c>
       <c r="B255" s="0" t="inlineStr">
         <is>
-          <t>宝宝数据已失效,请联系客服</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" s="0" t="inlineStr">
-        <is>
-          <t>PetSlotFull</t>
-        </is>
-      </c>
-      <c r="B256" s="0" t="inlineStr">
-        <is>
-          <t>可携带的宝宝数量已达上限</t>
-        </is>
-      </c>
-    </row>
+          <t>属性没有变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="256"/>
     <row r="257">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t>PetOwnerLevelNotEnough</t>
-        </is>
-      </c>
-      <c r="B257" s="0" t="inlineStr">
-        <is>
-          <t>主人等级不足,还不能携带这只宝宝</t>
+          <t>//pet_error base=26000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t>PetAlreadyActive</t>
+          <t>PetNotFound</t>
         </is>
       </c>
       <c r="B258" s="0" t="inlineStr">
         <is>
-          <t>这只宝宝已经在出战中</t>
+          <t>宝宝不存在</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="0" t="inlineStr">
         <is>
-          <t>PetNotActive</t>
+          <t>PetTableRowMissing</t>
         </is>
       </c>
       <c r="B259" s="0" t="inlineStr">
         <is>
-          <t>当前没有出战的宝宝</t>
+          <t>宝宝数据已失效,请联系客服</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t>PetSummonCooldown</t>
+          <t>PetSlotFull</t>
         </is>
       </c>
       <c r="B260" s="0" t="inlineStr">
         <is>
-          <t>操作太频繁,请稍后再试</t>
+          <t>可携带的宝宝数量已达上限</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t>PetNameInvalid</t>
+          <t>PetOwnerLevelNotEnough</t>
         </is>
       </c>
       <c r="B261" s="0" t="inlineStr">
         <is>
-          <t>宝宝名称不合法</t>
+          <t>主人等级不足,还不能携带这只宝宝</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="0" t="inlineStr">
         <is>
-          <t>PetInBattle</t>
+          <t>PetAlreadyActive</t>
         </is>
       </c>
       <c r="B262" s="0" t="inlineStr">
         <is>
-          <t>战斗中不能操作宝宝</t>
+          <t>这只宝宝已经在出战中</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t>PetPointsNotEnough</t>
+          <t>PetNotActive</t>
         </is>
       </c>
       <c r="B263" s="0" t="inlineStr">
         <is>
-          <t>宝宝剩余点数不足</t>
+          <t>当前没有出战的宝宝</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t>PetPointsCannotDecrease</t>
+          <t>PetSummonCooldown</t>
         </is>
       </c>
       <c r="B264" s="0" t="inlineStr">
         <is>
-          <t>已分配的点数不能减少,请使用洗点</t>
+          <t>操作太频繁,请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t>PetDimensionCapExceeded</t>
+          <t>PetNameInvalid</t>
         </is>
       </c>
       <c r="B265" s="0" t="inlineStr">
         <is>
-          <t>超过单项可分配上限</t>
+          <t>宝宝名称不合法</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t>PetDimensionNotFound</t>
+          <t>PetInBattle</t>
         </is>
       </c>
       <c r="B266" s="0" t="inlineStr">
         <is>
-          <t>宝宝属性维度不存在</t>
+          <t>战斗中不能操作宝宝</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t>PetGoldNotEnough</t>
+          <t>PetPointsNotEnough</t>
         </is>
       </c>
       <c r="B267" s="0" t="inlineStr">
         <is>
-          <t>金币不足</t>
+          <t>宝宝剩余点数不足</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t>PetNoAutoPlan</t>
+          <t>PetPointsCannotDecrease</t>
         </is>
       </c>
       <c r="B268" s="0" t="inlineStr">
         <is>
-          <t>没有可用的自动加点方案</t>
+          <t>已分配的点数不能减少,请使用洗点</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="0" t="inlineStr">
         <is>
-          <t>PetNothingToChange</t>
+          <t>PetDimensionCapExceeded</t>
         </is>
       </c>
       <c r="B269" s="0" t="inlineStr">
         <is>
-          <t>宝宝属性没有变化</t>
+          <t>超过单项可分配上限</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="0" t="inlineStr">
         <is>
+          <t>PetDimensionNotFound</t>
+        </is>
+      </c>
+      <c r="B270" s="0" t="inlineStr">
+        <is>
+          <t>宝宝属性维度不存在</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="0" t="inlineStr">
+        <is>
+          <t>PetGoldNotEnough</t>
+        </is>
+      </c>
+      <c r="B271" s="0" t="inlineStr">
+        <is>
+          <t>金币不足</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="0" t="inlineStr">
+        <is>
+          <t>PetNoAutoPlan</t>
+        </is>
+      </c>
+      <c r="B272" s="0" t="inlineStr">
+        <is>
+          <t>没有可用的自动加点方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="0" t="inlineStr">
+        <is>
+          <t>PetNothingToChange</t>
+        </is>
+      </c>
+      <c r="B273" s="0" t="inlineStr">
+        <is>
+          <t>宝宝属性没有变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="0" t="inlineStr">
+        <is>
           <t>PetIdGenerateFailed</t>
         </is>
       </c>
-      <c r="B270" s="0" t="inlineStr">
+      <c r="B274" s="0" t="inlineStr">
         <is>
           <t>宝宝创建失败,请稍后再试</t>
         </is>
       </c>
-      <c r="C270" s="0" t="n">
+      <c r="C274" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>//asset_error base=27000 width=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>AssetCurrencyInsufficient</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>货币不足</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>AssetBagFull</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>背包已满，请腾出空间，之后会重试发放；超过时限可能取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>AssetInBattle</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>战斗中暂不结算，稍后自动重试；超过时限可能取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>AssetFrozen</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>角色迁移中，稍后自动重试；超过时限可能取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>AssetInvalidBundle</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>资产指令无效</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>AssetBlocked</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>该资产当前被禁止获取</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>AssetPlayerNotHere</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>角色不在线，上线后重试；超过时限可能取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>AssetPartialApplied</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>资产只发放了一部分，已记录，将由客服补偿</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>AssetAuthFailed</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>资产指令校验失败</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP：每小时保存全部进度 2026-09-19 03:50:26 -04:00
</commit_message>
<xml_diff>
--- a/data/tip/Tip.xlsx
+++ b/data/tip/Tip.xlsx
@@ -1020,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C285"/>
+  <dimension ref="A1:C288"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="8" customWidth="1" style="2" min="3" max="3"/>
@@ -1714,100 +1714,115 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" ht="20" customHeight="1" s="2">
+    <row r="71">
       <c r="A71" s="0" t="inlineStr">
         <is>
+          <t>RoleNameInvalid</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t>角色名长度或字符不符合要求，仅限汉字、字母与数字</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t>RoleNameTaken</t>
+        </is>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t>该角色名已被使用，请换一个</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t>RoleNameSensitive</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t>角色名包含不允许使用的词语，请修改</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="n"/>
+    </row>
+    <row r="74" ht="20" customHeight="1" s="2">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
           <t>//scene_error base=3000 width=1000</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="20" customHeight="1" s="2">
-      <c r="A72" s="0" t="inlineStr">
+    <row r="75" ht="20" customHeight="1" s="2">
+      <c r="A75" s="0" t="inlineStr">
         <is>
           <t>EnterSceneNotFound</t>
         </is>
       </c>
-      <c r="B72" s="0" t="inlineStr">
+      <c r="B75" s="0" t="inlineStr">
         <is>
           <t>想进入的场景未找到</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="20" customHeight="1" s="2">
-      <c r="A73" s="0" t="inlineStr">
+    <row r="76" ht="20" customHeight="1" s="2">
+      <c r="A76" s="0" t="inlineStr">
         <is>
           <t>EnterSceneNotFull</t>
         </is>
       </c>
-      <c r="B73" s="0" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="0" t="inlineStr">
-        <is>
-          <t>EnterSceneMainFull</t>
-        </is>
-      </c>
-      <c r="B74" s="0" t="inlineStr">
-        <is>
-          <t>主场景已经满了</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="0" t="inlineStr">
-        <is>
-          <t>EnterNodeUnavailable</t>
-        </is>
-      </c>
-      <c r="B75" s="0" t="inlineStr">
-        <is>
-          <t>进入的游戏节点已不可用了</t>
-        </is>
-      </c>
-      <c r="C75" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="0" t="inlineStr">
-        <is>
-          <t>EnterSceneServerType</t>
-        </is>
-      </c>
-      <c r="B76" s="0" t="inlineStr">
-        <is>
-          <t>服务器未找到</t>
-        </is>
-      </c>
+      <c r="B76" s="0" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneParamError</t>
-        </is>
-      </c>
-      <c r="B77" s="0" t="inlineStr"/>
+          <t>EnterSceneMainFull</t>
+        </is>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t>主场景已经满了</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneSceneFull</t>
-        </is>
-      </c>
-      <c r="B78" s="0" t="inlineStr"/>
+          <t>EnterNodeUnavailable</t>
+        </is>
+      </c>
+      <c r="B78" s="0" t="inlineStr">
+        <is>
+          <t>进入的游戏节点已不可用了</t>
+        </is>
+      </c>
+      <c r="C78" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneSceneNotFound</t>
-        </is>
-      </c>
-      <c r="B79" s="0" t="inlineStr"/>
+          <t>EnterSceneServerType</t>
+        </is>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t>服务器未找到</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneYouInCurrentScene</t>
+          <t>EnterSceneParamError</t>
         </is>
       </c>
       <c r="B80" s="0" t="inlineStr"/>
@@ -1815,7 +1830,7 @@
     <row r="81">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneEnterCrossRoomScene</t>
+          <t>EnterSceneSceneFull</t>
         </is>
       </c>
       <c r="B81" s="0" t="inlineStr"/>
@@ -1823,18 +1838,15 @@
     <row r="82">
       <c r="A82" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneGsInfoNull</t>
+          <t>EnterSceneSceneNotFound</t>
         </is>
       </c>
       <c r="B82" s="0" t="inlineStr"/>
-      <c r="C82" s="0" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneGsFull</t>
+          <t>EnterSceneYouInCurrentScene</t>
         </is>
       </c>
       <c r="B83" s="0" t="inlineStr"/>
@@ -1842,26 +1854,26 @@
     <row r="84">
       <c r="A84" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneYourSceneIsNull</t>
+          <t>EnterSceneEnterCrossRoomScene</t>
         </is>
       </c>
       <c r="B84" s="0" t="inlineStr"/>
-      <c r="C84" s="0" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneChangeSceneOffLine</t>
+          <t>EnterSceneGsInfoNull</t>
         </is>
       </c>
       <c r="B85" s="0" t="inlineStr"/>
+      <c r="C85" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneChangingScene</t>
+          <t>EnterSceneGsFull</t>
         </is>
       </c>
       <c r="B86" s="0" t="inlineStr"/>
@@ -1869,26 +1881,26 @@
     <row r="87">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneChangingGs</t>
+          <t>EnterSceneYourSceneIsNull</t>
         </is>
       </c>
       <c r="B87" s="0" t="inlineStr"/>
+      <c r="C87" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="0" t="inlineStr">
         <is>
-          <t>ChangeScenePlayerQueueNotFound</t>
+          <t>EnterSceneChangeSceneOffLine</t>
         </is>
       </c>
       <c r="B88" s="0" t="inlineStr"/>
-      <c r="C88" s="0" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" s="0" t="inlineStr">
         <is>
-          <t>ChangeScenePlayerQueueFull</t>
+          <t>EnterSceneChangingScene</t>
         </is>
       </c>
       <c r="B89" s="0" t="inlineStr"/>
@@ -1896,18 +1908,15 @@
     <row r="90">
       <c r="A90" s="0" t="inlineStr">
         <is>
-          <t>ChangeScenePlayerQueueComponentGsNull</t>
+          <t>EnterSceneChangingGs</t>
         </is>
       </c>
       <c r="B90" s="0" t="inlineStr"/>
-      <c r="C90" s="0" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" s="0" t="inlineStr">
         <is>
-          <t>ChangeScenePlayerQueueComponentEmpty</t>
+          <t>ChangeScenePlayerQueueNotFound</t>
         </is>
       </c>
       <c r="B91" s="0" t="inlineStr"/>
@@ -1918,7 +1927,7 @@
     <row r="92">
       <c r="A92" s="0" t="inlineStr">
         <is>
-          <t>ChangeSceneEnQueueNotSameGs</t>
+          <t>ChangeScenePlayerQueueFull</t>
         </is>
       </c>
       <c r="B92" s="0" t="inlineStr"/>
@@ -1926,78 +1935,69 @@
     <row r="93">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t>InvalidEnterSceneParameters</t>
+          <t>ChangeScenePlayerQueueComponentGsNull</t>
         </is>
       </c>
       <c r="B93" s="0" t="inlineStr"/>
+      <c r="C93" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="0" t="inlineStr">
         <is>
-          <t>CheckEnterSceneCreator</t>
+          <t>ChangeScenePlayerQueueComponentEmpty</t>
         </is>
       </c>
       <c r="B94" s="0" t="inlineStr"/>
+      <c r="C94" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="0" t="inlineStr">
         <is>
-          <t>EnterSceneFailed</t>
+          <t>ChangeSceneEnQueueNotSameGs</t>
         </is>
       </c>
       <c r="B95" s="0" t="inlineStr"/>
-      <c r="C95" s="0" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="96">
       <c r="A96" s="0" t="inlineStr">
         <is>
-          <t>ZoneTravelTargetZoneNotFound</t>
-        </is>
-      </c>
-      <c r="B96" s="0" t="inlineStr">
-        <is>
-          <t>目标区服不存在</t>
-        </is>
-      </c>
-      <c r="C96" s="0" t="n"/>
+          <t>InvalidEnterSceneParameters</t>
+        </is>
+      </c>
+      <c r="B96" s="0" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="0" t="inlineStr">
         <is>
-          <t>ZoneTravelInBattle</t>
-        </is>
-      </c>
-      <c r="B97" s="0" t="inlineStr">
-        <is>
-          <t>战斗中不能传送</t>
-        </is>
-      </c>
-      <c r="C97" s="0" t="n"/>
+          <t>CheckEnterSceneCreator</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="0" t="inlineStr">
         <is>
-          <t>ZoneTravelInTeam</t>
-        </is>
-      </c>
-      <c r="B98" s="0" t="inlineStr">
-        <is>
-          <t>组队中不能传送</t>
-        </is>
-      </c>
-      <c r="C98" s="0" t="n"/>
+          <t>EnterSceneFailed</t>
+        </is>
+      </c>
+      <c r="B98" s="0" t="inlineStr"/>
+      <c r="C98" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="0" t="inlineStr">
         <is>
-          <t>ZoneTravelTargetBusy</t>
+          <t>ZoneTravelTargetZoneNotFound</t>
         </is>
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>目标区服繁忙,请稍后再试</t>
+          <t>目标区服不存在</t>
         </is>
       </c>
       <c r="C99" s="0" t="n"/>
@@ -2005,158 +2005,161 @@
     <row r="100">
       <c r="A100" s="0" t="inlineStr">
         <is>
-          <t>//team_error base=4000 width=1000</t>
-        </is>
-      </c>
+          <t>ZoneTravelInBattle</t>
+        </is>
+      </c>
+      <c r="B100" s="0" t="inlineStr">
+        <is>
+          <t>战斗中不能传送</t>
+        </is>
+      </c>
+      <c r="C100" s="0" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="0" t="inlineStr">
         <is>
-          <t>TeamNotInApplicants</t>
+          <t>ZoneTravelInTeam</t>
         </is>
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
-        </is>
-      </c>
+          <t>组队中不能传送</t>
+        </is>
+      </c>
+      <c r="C101" s="0" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="0" t="inlineStr">
         <is>
-          <t>TeamPlayerId</t>
+          <t>ZoneTravelTargetBusy</t>
         </is>
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t>玩家 ID 无效</t>
-        </is>
-      </c>
+          <t>目标区服繁忙,请稍后再试</t>
+        </is>
+      </c>
+      <c r="C102" s="0" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="0" t="inlineStr">
         <is>
-          <t>TeamMembersFull</t>
-        </is>
-      </c>
-      <c r="B103" s="0" t="inlineStr">
-        <is>
-          <t>队伍人数已满</t>
+          <t>//team_error base=4000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberInTeam</t>
+          <t>TeamNotInApplicants</t>
         </is>
       </c>
       <c r="B104" s="0" t="inlineStr">
         <is>
-          <t>对方已经在队伍中</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberNotInTeam</t>
+          <t>TeamPlayerId</t>
         </is>
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t>对方不在你的队伍中</t>
+          <t>玩家 ID 无效</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="0" t="inlineStr">
         <is>
-          <t>TeamKickSelf</t>
+          <t>TeamMembersFull</t>
         </is>
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t>不能把自己踢出队伍</t>
+          <t>队伍人数已满</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="0" t="inlineStr">
         <is>
-          <t>TeamKickNotLeader</t>
+          <t>TeamMemberInTeam</t>
         </is>
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t>只有队长可以踢人</t>
+          <t>对方已经在队伍中</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="0" t="inlineStr">
         <is>
-          <t>TeamAppointSelf</t>
+          <t>TeamMemberNotInTeam</t>
         </is>
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t>你已经是队长了</t>
+          <t>对方不在你的队伍中</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="0" t="inlineStr">
         <is>
-          <t>TeamAppointLeaderNotLeader</t>
+          <t>TeamKickSelf</t>
         </is>
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t>只有队长可以转让队长</t>
+          <t>不能把自己踢出队伍</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="0" t="inlineStr">
         <is>
-          <t>TeamFull</t>
+          <t>TeamKickNotLeader</t>
         </is>
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
+          <t>只有队长可以踢人</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="0" t="inlineStr">
         <is>
-          <t>TeamInApplicantList</t>
+          <t>TeamAppointSelf</t>
         </is>
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
+          <t>你已经是队长了</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="0" t="inlineStr">
         <is>
-          <t>TeamNotInApplicantList</t>
+          <t>TeamAppointLeaderNotLeader</t>
         </is>
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t>该申请已失效</t>
+          <t>只有队长可以转让队长</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="0" t="inlineStr">
         <is>
-          <t>TeamListMaxSize</t>
+          <t>TeamFull</t>
         </is>
       </c>
       <c r="B113" s="0" t="inlineStr">
@@ -2168,31 +2171,31 @@
     <row r="114">
       <c r="A114" s="0" t="inlineStr">
         <is>
-          <t>TeamHasNotTeamId</t>
+          <t>TeamInApplicantList</t>
         </is>
       </c>
       <c r="B114" s="0" t="inlineStr">
         <is>
-          <t>你还没有队伍</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="0" t="inlineStr">
         <is>
-          <t>TeamDismissNotLeader</t>
+          <t>TeamNotInApplicantList</t>
         </is>
       </c>
       <c r="B115" s="0" t="inlineStr">
         <is>
-          <t>只有队长可以解散队伍</t>
+          <t>该申请已失效</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberListFull</t>
+          <t>TeamListMaxSize</t>
         </is>
       </c>
       <c r="B116" s="0" t="inlineStr">
@@ -2204,232 +2207,241 @@
     <row r="117">
       <c r="A117" s="0" t="inlineStr">
         <is>
-          <t>TeamCreateTeamMaxMemberSize</t>
+          <t>TeamHasNotTeamId</t>
         </is>
       </c>
       <c r="B117" s="0" t="inlineStr">
         <is>
-          <t>(保留)</t>
+          <t>你还没有队伍</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="0" t="inlineStr">
         <is>
-          <t>TeamPlayerNotFound</t>
+          <t>TeamDismissNotLeader</t>
         </is>
       </c>
       <c r="B118" s="0" t="inlineStr">
         <is>
-          <t>找不到该玩家</t>
+          <t>只有队长可以解散队伍</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="0" t="inlineStr">
         <is>
-          <t>TeamNotLeader</t>
+          <t>TeamMemberListFull</t>
         </is>
       </c>
       <c r="B119" s="0" t="inlineStr">
         <is>
-          <t>只有队长可以执行此操作</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="0" t="inlineStr">
         <is>
-          <t>TeamHomeZoneUnknown</t>
+          <t>TeamCreateTeamMaxMemberSize</t>
         </is>
       </c>
       <c r="B120" s="0" t="inlineStr">
         <is>
-          <t>角色区服信息异常，请重新登录</t>
+          <t>(保留)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="0" t="inlineStr">
         <is>
-          <t>TeamCrossZoneDenied</t>
+          <t>TeamPlayerNotFound</t>
         </is>
       </c>
       <c r="B121" s="0" t="inlineStr">
         <is>
-          <t>不能与其他区服的玩家组队</t>
+          <t>找不到该玩家</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="0" t="inlineStr">
         <is>
-          <t>TeamInviteNotFound</t>
+          <t>TeamNotLeader</t>
         </is>
       </c>
       <c r="B122" s="0" t="inlineStr">
         <is>
-          <t>邀请已失效</t>
+          <t>只有队长可以执行此操作</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="0" t="inlineStr">
         <is>
-          <t>TeamInviteLimit</t>
+          <t>TeamHomeZoneUnknown</t>
         </is>
       </c>
       <c r="B123" s="0" t="inlineStr">
         <is>
-          <t>对方待处理的邀请过多，请稍后再试</t>
+          <t>角色区服信息异常，请重新登录</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="0" t="inlineStr">
         <is>
-          <t>TeamInMatch</t>
+          <t>TeamCrossZoneDenied</t>
         </is>
       </c>
       <c r="B124" s="0" t="inlineStr">
         <is>
-          <t>队伍正在进入战斗，请稍候</t>
+          <t>不能与其他区服的玩家组队</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberOffline</t>
+          <t>TeamInviteNotFound</t>
         </is>
       </c>
       <c r="B125" s="0" t="inlineStr">
         <is>
-          <t>有队员不在线</t>
+          <t>邀请已失效</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberInBattle</t>
+          <t>TeamInviteLimit</t>
         </is>
       </c>
       <c r="B126" s="0" t="inlineStr">
         <is>
-          <t>有队员正在战斗中</t>
+          <t>对方待处理的邀请过多，请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="0" t="inlineStr">
         <is>
-          <t>TeamMemberNotReady</t>
+          <t>TeamInMatch</t>
         </is>
       </c>
       <c r="B127" s="0" t="inlineStr">
         <is>
-          <t>有队员暂时无法开战</t>
+          <t>队伍正在进入战斗，请稍候</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="0" t="inlineStr">
         <is>
-          <t>TeamDungeonNotOpen</t>
+          <t>TeamMemberOffline</t>
         </is>
       </c>
       <c r="B128" s="0" t="inlineStr">
         <is>
-          <t>该副本未开放组队</t>
+          <t>有队员不在线</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="0" t="inlineStr">
         <is>
-          <t>TeamSizeExceeded</t>
+          <t>TeamMemberInBattle</t>
         </is>
       </c>
       <c r="B129" s="0" t="inlineStr">
         <is>
-          <t>队伍人数超过该副本上限</t>
+          <t>有队员正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="0" t="inlineStr">
         <is>
-          <t>TeamStateChanged</t>
+          <t>TeamMemberNotReady</t>
         </is>
       </c>
       <c r="B130" s="0" t="inlineStr">
         <is>
-          <t>队伍状态已变化，请重试</t>
+          <t>有队员暂时无法开战</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="0" t="inlineStr">
         <is>
-          <t>TeamInternal</t>
+          <t>TeamDungeonNotOpen</t>
         </is>
       </c>
       <c r="B131" s="0" t="inlineStr">
         <is>
-          <t>服务器繁忙，请稍后再试</t>
-        </is>
-      </c>
-      <c r="C131" s="0" t="n">
-        <v>1</v>
+          <t>该副本未开放组队</t>
+        </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="0" t="inlineStr">
         <is>
-          <t>//mission_error base=5000 width=1000</t>
+          <t>TeamSizeExceeded</t>
+        </is>
+      </c>
+      <c r="B132" s="0" t="inlineStr">
+        <is>
+          <t>队伍人数超过该副本上限</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="0" t="inlineStr">
         <is>
-          <t>MissionTypeAlreadyExists</t>
-        </is>
-      </c>
-      <c r="B133" s="0" t="inlineStr"/>
+          <t>TeamStateChanged</t>
+        </is>
+      </c>
+      <c r="B133" s="0" t="inlineStr">
+        <is>
+          <t>队伍状态已变化，请重试</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="0" t="inlineStr">
         <is>
-          <t>MissionAlreadyCompleted</t>
-        </is>
-      </c>
-      <c r="B134" s="0" t="inlineStr"/>
+          <t>TeamInternal</t>
+        </is>
+      </c>
+      <c r="B134" s="0" t="inlineStr">
+        <is>
+          <t>服务器繁忙，请稍后再试</t>
+        </is>
+      </c>
+      <c r="C134" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="0" t="inlineStr">
         <is>
-          <t>MissionIdNotInRewardList</t>
-        </is>
-      </c>
-      <c r="B135" s="0" t="inlineStr"/>
+          <t>//mission_error base=5000 width=1000</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="0" t="inlineStr">
         <is>
-          <t>PlayerMissionComponentNotFound</t>
+          <t>MissionTypeAlreadyExists</t>
         </is>
       </c>
       <c r="B136" s="0" t="inlineStr"/>
-      <c r="C136" s="0" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="137">
       <c r="A137" s="0" t="inlineStr">
         <is>
-          <t>MissionIdRepeated</t>
+          <t>MissionAlreadyCompleted</t>
         </is>
       </c>
       <c r="B137" s="0" t="inlineStr"/>
@@ -2437,7 +2449,7 @@
     <row r="138">
       <c r="A138" s="0" t="inlineStr">
         <is>
-          <t>ConditionIdOutOfRange</t>
+          <t>MissionIdNotInRewardList</t>
         </is>
       </c>
       <c r="B138" s="0" t="inlineStr"/>
@@ -2445,22 +2457,26 @@
     <row r="139">
       <c r="A139" s="0" t="inlineStr">
         <is>
-          <t>MissionNotInProgress</t>
+          <t>PlayerMissionComponentNotFound</t>
         </is>
       </c>
       <c r="B139" s="0" t="inlineStr"/>
+      <c r="C139" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="0" t="inlineStr">
         <is>
-          <t>//bag_error base=6000 width=1000</t>
-        </is>
-      </c>
+          <t>MissionIdRepeated</t>
+        </is>
+      </c>
+      <c r="B140" s="0" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="0" t="inlineStr">
         <is>
-          <t>BagDeleteItemFindGuid</t>
+          <t>ConditionIdOutOfRange</t>
         </is>
       </c>
       <c r="B141" s="0" t="inlineStr"/>
@@ -2468,7 +2484,7 @@
     <row r="142">
       <c r="A142" s="0" t="inlineStr">
         <is>
-          <t>BagDeleteItemAlreadyHasGuid</t>
+          <t>MissionNotInProgress</t>
         </is>
       </c>
       <c r="B142" s="0" t="inlineStr"/>
@@ -2476,18 +2492,14 @@
     <row r="143">
       <c r="A143" s="0" t="inlineStr">
         <is>
-          <t>BagAddItemHasNotBaseComponent</t>
-        </is>
-      </c>
-      <c r="B143" s="0" t="inlineStr"/>
-      <c r="C143" s="0" t="n">
-        <v>1</v>
+          <t>//bag_error base=6000 width=1000</t>
+        </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="0" t="inlineStr">
         <is>
-          <t>BagAddItemInvalidGuid</t>
+          <t>BagDeleteItemFindGuid</t>
         </is>
       </c>
       <c r="B144" s="0" t="inlineStr"/>
@@ -2495,7 +2507,7 @@
     <row r="145">
       <c r="A145" s="0" t="inlineStr">
         <is>
-          <t>BagAddItemInvalidParam</t>
+          <t>BagDeleteItemAlreadyHasGuid</t>
         </is>
       </c>
       <c r="B145" s="0" t="inlineStr"/>
@@ -2503,15 +2515,18 @@
     <row r="146">
       <c r="A146" s="0" t="inlineStr">
         <is>
-          <t>BagAddItemBagFull</t>
+          <t>BagAddItemHasNotBaseComponent</t>
         </is>
       </c>
       <c r="B146" s="0" t="inlineStr"/>
+      <c r="C146" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="0" t="inlineStr">
         <is>
-          <t>BagItemNotStacked</t>
+          <t>BagAddItemInvalidGuid</t>
         </is>
       </c>
       <c r="B147" s="0" t="inlineStr"/>
@@ -2519,7 +2534,7 @@
     <row r="148">
       <c r="A148" s="0" t="inlineStr">
         <is>
-          <t>BagInsufficientItems</t>
+          <t>BagAddItemInvalidParam</t>
         </is>
       </c>
       <c r="B148" s="0" t="inlineStr"/>
@@ -2527,7 +2542,7 @@
     <row r="149">
       <c r="A149" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemPos</t>
+          <t>BagAddItemBagFull</t>
         </is>
       </c>
       <c r="B149" s="0" t="inlineStr"/>
@@ -2535,7 +2550,7 @@
     <row r="150">
       <c r="A150" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemConfig</t>
+          <t>BagItemNotStacked</t>
         </is>
       </c>
       <c r="B150" s="0" t="inlineStr"/>
@@ -2543,7 +2558,7 @@
     <row r="151">
       <c r="A151" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemGuid</t>
+          <t>BagInsufficientItems</t>
         </is>
       </c>
       <c r="B151" s="0" t="inlineStr"/>
@@ -2551,7 +2566,7 @@
     <row r="152">
       <c r="A152" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemFindItem</t>
+          <t>BagDelItemPos</t>
         </is>
       </c>
       <c r="B152" s="0" t="inlineStr"/>
@@ -2559,7 +2574,7 @@
     <row r="153">
       <c r="A153" s="0" t="inlineStr">
         <is>
-          <t>BagDelItemSize</t>
+          <t>BagDelItemConfig</t>
         </is>
       </c>
       <c r="B153" s="0" t="inlineStr"/>
@@ -2567,7 +2582,7 @@
     <row r="154">
       <c r="A154" s="0" t="inlineStr">
         <is>
-          <t>BagItemDeletionSizeMismatch</t>
+          <t>BagDelItemGuid</t>
         </is>
       </c>
       <c r="B154" s="0" t="inlineStr"/>
@@ -2575,7 +2590,7 @@
     <row r="155">
       <c r="A155" s="0" t="inlineStr">
         <is>
-          <t>BagInsufficientBagSpace</t>
+          <t>BagDelItemFindItem</t>
         </is>
       </c>
       <c r="B155" s="0" t="inlineStr"/>
@@ -2583,1445 +2598,1470 @@
     <row r="156">
       <c r="A156" s="0" t="inlineStr">
         <is>
-          <t>//skill_error base=7000 width=1000</t>
-        </is>
-      </c>
+          <t>BagDelItemSize</t>
+        </is>
+      </c>
+      <c r="B156" s="0" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="0" t="inlineStr">
         <is>
-          <t>SkillUnInterruptible</t>
-        </is>
-      </c>
-      <c r="B157" s="0" t="inlineStr">
-        <is>
-          <t>技能不能被打断</t>
-        </is>
-      </c>
+          <t>BagItemDeletionSizeMismatch</t>
+        </is>
+      </c>
+      <c r="B157" s="0" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="0" t="inlineStr">
         <is>
-          <t>SkillInvalidTargetId</t>
-        </is>
-      </c>
-      <c r="B158" s="0" t="inlineStr">
-        <is>
-          <t>目标id错误</t>
-        </is>
-      </c>
+          <t>BagInsufficientBagSpace</t>
+        </is>
+      </c>
+      <c r="B158" s="0" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="0" t="inlineStr">
         <is>
-          <t>SkillInvalidTarget</t>
-        </is>
-      </c>
-      <c r="B159" s="0" t="inlineStr">
-        <is>
-          <t>未找到释放目标</t>
+          <t>//skill_error base=7000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="0" t="inlineStr">
         <is>
-          <t>SkillCooldownNotReady</t>
+          <t>SkillUnInterruptible</t>
         </is>
       </c>
       <c r="B160" s="0" t="inlineStr">
         <is>
-          <t>技能冷却尚未完成，无法使用技能</t>
+          <t>技能不能被打断</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="0" t="inlineStr">
         <is>
-          <t>SkillCannotBeCastInCurrentState</t>
+          <t>SkillInvalidTargetId</t>
         </is>
       </c>
       <c r="B161" s="0" t="inlineStr">
         <is>
-          <t>当前状态不能释放该技能</t>
+          <t>目标id错误</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="0" t="inlineStr">
         <is>
-          <t>SkillCannotBeCastSilenceRestriction</t>
+          <t>SkillInvalidTarget</t>
         </is>
       </c>
       <c r="B162" s="0" t="inlineStr">
         <is>
-          <t>当前沉默状态不能释放该技能</t>
+          <t>未找到释放目标</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="0" t="inlineStr">
         <is>
-          <t>SkillCannotBeCastStunRestriction</t>
+          <t>SkillCooldownNotReady</t>
         </is>
       </c>
       <c r="B163" s="0" t="inlineStr">
         <is>
-          <t>当前眩晕状态不能释放该技能</t>
+          <t>技能冷却尚未完成，无法使用技能</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="0" t="inlineStr">
         <is>
-          <t>//buff_error base=8000 width=1000</t>
+          <t>SkillCannotBeCastInCurrentState</t>
+        </is>
+      </c>
+      <c r="B164" s="0" t="inlineStr">
+        <is>
+          <t>当前状态不能释放该技能</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="0" t="inlineStr">
         <is>
-          <t>BuffMaxBuffStack</t>
+          <t>SkillCannotBeCastSilenceRestriction</t>
         </is>
       </c>
       <c r="B165" s="0" t="inlineStr">
         <is>
-          <t>buff层数已经最大</t>
+          <t>当前沉默状态不能释放该技能</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="0" t="inlineStr">
         <is>
-          <t>BuffTargetImmuneToBuff</t>
+          <t>SkillCannotBeCastStunRestriction</t>
         </is>
       </c>
       <c r="B166" s="0" t="inlineStr">
         <is>
-          <t>目标免疫buff</t>
+          <t>当前眩晕状态不能释放该技能</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="0" t="inlineStr">
         <is>
-          <t>//entity_error base=9000 width=1000</t>
+          <t>//buff_error base=8000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="0" t="inlineStr">
         <is>
-          <t>EntityTransformNotFound</t>
+          <t>BuffMaxBuffStack</t>
         </is>
       </c>
       <c r="B168" s="0" t="inlineStr">
         <is>
-          <t>未找到实体的Transfor组件</t>
-        </is>
-      </c>
-      <c r="C168" s="0" t="n">
-        <v>1</v>
+          <t>buff层数已经最大</t>
+        </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="0" t="inlineStr">
         <is>
-          <t>//actor_action_error base=10000 width=1000</t>
+          <t>BuffTargetImmuneToBuff</t>
+        </is>
+      </c>
+      <c r="B169" s="0" t="inlineStr">
+        <is>
+          <t>目标免疫buff</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="0" t="inlineStr">
         <is>
-          <t>ActorActionStateActionCannotBePerformedWhileInTeamFollowMode</t>
-        </is>
-      </c>
-      <c r="B170" s="0" t="inlineStr">
-        <is>
-          <t>正在组队跟随中</t>
+          <t>//entity_error base=9000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="0" t="inlineStr">
         <is>
-          <t>//mount_error base=11000 width=1000</t>
-        </is>
+          <t>EntityTransformNotFound</t>
+        </is>
+      </c>
+      <c r="B171" s="0" t="inlineStr">
+        <is>
+          <t>未找到实体的Transfor组件</t>
+        </is>
+      </c>
+      <c r="C171" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="0" t="inlineStr">
         <is>
-          <t>MountNotMounted</t>
-        </is>
-      </c>
-      <c r="B172" s="0" t="inlineStr">
-        <is>
-          <t>当前不在坐骑上</t>
+          <t>//actor_action_error base=10000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="0" t="inlineStr">
         <is>
-          <t>//reward_error base=12000 width=1000</t>
+          <t>ActorActionStateActionCannotBePerformedWhileInTeamFollowMode</t>
+        </is>
+      </c>
+      <c r="B173" s="0" t="inlineStr">
+        <is>
+          <t>正在组队跟随中</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="0" t="inlineStr">
         <is>
-          <t>RewardAlreadyClaimed</t>
-        </is>
-      </c>
-      <c r="B174" s="0" t="inlineStr">
-        <is>
-          <t>该奖励已经领取过了</t>
+          <t>//mount_error base=11000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="0" t="inlineStr">
         <is>
-          <t>//cross_server_error base=13000 width=1000</t>
+          <t>MountNotMounted</t>
+        </is>
+      </c>
+      <c r="B175" s="0" t="inlineStr">
+        <is>
+          <t>当前不在坐骑上</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="0" t="inlineStr">
         <is>
-          <t>SceneTransferInProgress</t>
-        </is>
-      </c>
-      <c r="B176" s="0" t="inlineStr"/>
+          <t>//reward_error base=12000 width=1000</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t>//guild_error base=14000 width=1000</t>
+          <t>RewardAlreadyClaimed</t>
+        </is>
+      </c>
+      <c r="B177" s="0" t="inlineStr">
+        <is>
+          <t>该奖励已经领取过了</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t>GuildAlreadyInGuild</t>
-        </is>
-      </c>
-      <c r="B178" s="0" t="inlineStr">
-        <is>
-          <t>已加入公会</t>
+          <t>//cross_server_error base=13000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t>GuildNotFound</t>
-        </is>
-      </c>
-      <c r="B179" s="0" t="inlineStr">
-        <is>
-          <t>公会不存在</t>
-        </is>
-      </c>
+          <t>SceneTransferInProgress</t>
+        </is>
+      </c>
+      <c r="B179" s="0" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t>GuildNotInGuild</t>
-        </is>
-      </c>
-      <c r="B180" s="0" t="inlineStr">
-        <is>
-          <t>尚未加入公会</t>
+          <t>//guild_error base=14000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t>GuildFull</t>
+          <t>GuildAlreadyInGuild</t>
         </is>
       </c>
       <c r="B181" s="0" t="inlineStr">
         <is>
-          <t>公会人数已满</t>
+          <t>已加入公会</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t>GuildLeaderCantLeave</t>
+          <t>GuildNotFound</t>
         </is>
       </c>
       <c r="B182" s="0" t="inlineStr">
         <is>
-          <t>会长不能退出公会</t>
+          <t>公会不存在</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t>GuildNotLeader</t>
+          <t>GuildNotInGuild</t>
         </is>
       </c>
       <c r="B183" s="0" t="inlineStr">
         <is>
-          <t>只有会长可以执行该操作</t>
+          <t>尚未加入公会</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t>GuildNoPermission</t>
+          <t>GuildFull</t>
         </is>
       </c>
       <c r="B184" s="0" t="inlineStr">
         <is>
-          <t>权限不足</t>
+          <t>公会人数已满</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t>GuildNotRanked</t>
+          <t>GuildLeaderCantLeave</t>
         </is>
       </c>
       <c r="B185" s="0" t="inlineStr">
         <is>
-          <t>暂未上榜</t>
+          <t>会长不能退出公会</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t>GuildIdGenUnavailable</t>
+          <t>GuildNotLeader</t>
         </is>
       </c>
       <c r="B186" s="0" t="inlineStr">
         <is>
-          <t>服务繁忙，请稍后重试</t>
-        </is>
-      </c>
-      <c r="C186" s="0" t="n">
-        <v>1</v>
+          <t>只有会长可以执行该操作</t>
+        </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="0" t="inlineStr">
         <is>
-          <t>GuildNameInvalid</t>
+          <t>GuildNoPermission</t>
         </is>
       </c>
       <c r="B187" s="0" t="inlineStr">
         <is>
-          <t>公会名称无效（1-24 个字，不能包含控制字符）</t>
+          <t>权限不足</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="0" t="inlineStr">
         <is>
-          <t>GuildNameTaken</t>
+          <t>GuildNotRanked</t>
         </is>
       </c>
       <c r="B188" s="0" t="inlineStr">
         <is>
-          <t>公会名称已被使用</t>
+          <t>暂未上榜</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="0" t="inlineStr">
         <is>
-          <t>GuildAnnouncementTooLong</t>
+          <t>GuildIdGenUnavailable</t>
         </is>
       </c>
       <c r="B189" s="0" t="inlineStr">
         <is>
-          <t>公会公告过长</t>
-        </is>
+          <t>服务繁忙，请稍后重试</t>
+        </is>
+      </c>
+      <c r="C189" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="0" t="inlineStr">
         <is>
-          <t>GuildHomeZoneUnknown</t>
+          <t>GuildNameInvalid</t>
         </is>
       </c>
       <c r="B190" s="0" t="inlineStr">
         <is>
-          <t>角色归属区服未确认，暂时无法使用公会</t>
+          <t>公会名称无效（1-24 个字，不能包含控制字符）</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t>GuildZoneMerging</t>
+          <t>GuildNameTaken</t>
         </is>
       </c>
       <c r="B191" s="0" t="inlineStr">
         <is>
-          <t>区服合并维护中，帮会操作暂停，请稍后再试</t>
+          <t>公会名称已被使用</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t>GuildTargetNotMember</t>
+          <t>GuildAnnouncementTooLong</t>
         </is>
       </c>
       <c r="B192" s="0" t="inlineStr">
         <is>
-          <t>对方已不在本帮会</t>
+          <t>公会公告过长</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t>GuildCannotTargetSelf</t>
+          <t>GuildHomeZoneUnknown</t>
         </is>
       </c>
       <c r="B193" s="0" t="inlineStr">
         <is>
-          <t>不能对自己执行此操作</t>
+          <t>角色归属区服未确认，暂时无法使用公会</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t>GuildRankTooLow</t>
+          <t>GuildZoneMerging</t>
         </is>
       </c>
       <c r="B194" s="0" t="inlineStr">
         <is>
-          <t>帮会职位不足，无法执行此操作</t>
+          <t>区服合并维护中，帮会操作暂停，请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="0" t="inlineStr">
         <is>
-          <t>GuildOfficerLimit</t>
+          <t>GuildTargetNotMember</t>
         </is>
       </c>
       <c r="B195" s="0" t="inlineStr">
         <is>
-          <t>长老人数已达当前帮会等级上限</t>
+          <t>对方已不在本帮会</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t>GuildApplicationNotFound</t>
+          <t>GuildCannotTargetSelf</t>
         </is>
       </c>
       <c r="B196" s="0" t="inlineStr">
         <is>
-          <t>入帮申请不存在或已失效</t>
+          <t>不能对自己执行此操作</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t>GuildApplicationLimit</t>
+          <t>GuildRankTooLow</t>
         </is>
       </c>
       <c r="B197" s="0" t="inlineStr">
         <is>
-          <t>同时进行中的入帮申请已达上限</t>
+          <t>帮会职位不足，无法执行此操作</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t>GuildApplicationQueueFull</t>
+          <t>GuildOfficerLimit</t>
         </is>
       </c>
       <c r="B198" s="0" t="inlineStr">
         <is>
-          <t>该帮会待审申请已满，请稍后再试</t>
+          <t>长老人数已达当前帮会等级上限</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t>GuildBusyRetry</t>
+          <t>GuildApplicationNotFound</t>
         </is>
       </c>
       <c r="B199" s="0" t="inlineStr">
         <is>
-          <t>帮会操作繁忙，请稍后重试</t>
+          <t>入帮申请不存在或已失效</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t>//friend_error base=15000 width=1000</t>
+          <t>GuildApplicationLimit</t>
+        </is>
+      </c>
+      <c r="B200" s="0" t="inlineStr">
+        <is>
+          <t>同时进行中的入帮申请已达上限</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t>FriendCannotAddSelf</t>
+          <t>GuildApplicationQueueFull</t>
         </is>
       </c>
       <c r="B201" s="0" t="inlineStr">
         <is>
-          <t>不能添加自己为好友</t>
+          <t>该帮会待审申请已满，请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t>FriendAlreadyFriends</t>
+          <t>GuildBusyRetry</t>
         </is>
       </c>
       <c r="B202" s="0" t="inlineStr">
         <is>
-          <t>你们已经是好友了</t>
+          <t>帮会操作繁忙，请稍后重试</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>FriendListFull</t>
-        </is>
-      </c>
-      <c r="B203" s="0" t="inlineStr">
-        <is>
-          <t>好友列表已满</t>
+          <t>//friend_error base=15000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t>FriendRequestAlreadySent</t>
+          <t>FriendCannotAddSelf</t>
         </is>
       </c>
       <c r="B204" s="0" t="inlineStr">
         <is>
-          <t>已发送过好友申请</t>
+          <t>不能添加自己为好友</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t>FriendTargetListFull</t>
+          <t>FriendAlreadyFriends</t>
         </is>
       </c>
       <c r="B205" s="0" t="inlineStr">
         <is>
-          <t>对方好友列表已满</t>
+          <t>你们已经是好友了</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t>FriendNoPendingRequest</t>
+          <t>FriendListFull</t>
         </is>
       </c>
       <c r="B206" s="0" t="inlineStr">
         <is>
-          <t>没有待处理的好友申请</t>
+          <t>好友列表已满</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t>FriendTooManyPending</t>
+          <t>FriendRequestAlreadySent</t>
         </is>
       </c>
       <c r="B207" s="0" t="inlineStr">
         <is>
-          <t>待处理的申请过多</t>
+          <t>已发送过好友申请</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t>//match_error base=16000 width=1000</t>
+          <t>FriendTargetListFull</t>
+        </is>
+      </c>
+      <c r="B208" s="0" t="inlineStr">
+        <is>
+          <t>对方好友列表已满</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t>MatchInBattle</t>
+          <t>FriendNoPendingRequest</t>
         </is>
       </c>
       <c r="B209" s="0" t="inlineStr">
         <is>
-          <t>你正在战斗中</t>
+          <t>没有待处理的好友申请</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t>MatchAlreadyQueued</t>
+          <t>FriendTooManyPending</t>
         </is>
       </c>
       <c r="B210" s="0" t="inlineStr">
         <is>
-          <t>已在匹配队列中</t>
+          <t>待处理的申请过多</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t>MatchModeNotOpen</t>
-        </is>
-      </c>
-      <c r="B211" s="0" t="inlineStr">
-        <is>
-          <t>该匹配模式暂未开放</t>
+          <t>//match_error base=16000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t>MatchTeamSizeNotConfigured</t>
+          <t>MatchInBattle</t>
         </is>
       </c>
       <c r="B212" s="0" t="inlineStr">
         <is>
-          <t>队伍人数未配置</t>
+          <t>你正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t>MatchInternal</t>
+          <t>MatchAlreadyQueued</t>
         </is>
       </c>
       <c r="B213" s="0" t="inlineStr">
         <is>
-          <t>服务繁忙，请稍后重试</t>
-        </is>
-      </c>
-      <c r="C213" s="0" t="n"/>
+          <t>已在匹配队列中</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t>MatchTicketMismatch</t>
+          <t>MatchModeNotOpen</t>
         </is>
       </c>
       <c r="B214" s="0" t="inlineStr">
         <is>
-          <t>匹配凭据不匹配</t>
+          <t>该匹配模式暂未开放</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t>MatchCancelTooLate</t>
+          <t>MatchTeamSizeNotConfigured</t>
         </is>
       </c>
       <c r="B215" s="0" t="inlineStr">
         <is>
-          <t>匹配已开始，无法取消</t>
+          <t>队伍人数未配置</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeSelf</t>
+          <t>MatchInternal</t>
         </is>
       </c>
       <c r="B216" s="0" t="inlineStr">
         <is>
-          <t>不能挑战自己</t>
-        </is>
-      </c>
+          <t>服务繁忙，请稍后重试</t>
+        </is>
+      </c>
+      <c r="C216" s="0" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeTargetOffline</t>
+          <t>MatchTicketMismatch</t>
         </is>
       </c>
       <c r="B217" s="0" t="inlineStr">
         <is>
-          <t>对方不在线</t>
+          <t>匹配凭据不匹配</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeTargetBusy</t>
+          <t>MatchCancelTooLate</t>
         </is>
       </c>
       <c r="B218" s="0" t="inlineStr">
         <is>
-          <t>对方正在战斗中</t>
+          <t>匹配已开始，无法取消</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeSelfBusy</t>
+          <t>MatchChallengeSelf</t>
         </is>
       </c>
       <c r="B219" s="0" t="inlineStr">
         <is>
-          <t>你正在战斗中</t>
+          <t>不能挑战自己</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengePending</t>
+          <t>MatchChallengeTargetOffline</t>
         </is>
       </c>
       <c r="B220" s="0" t="inlineStr">
         <is>
-          <t>已有待应答的挑战</t>
+          <t>对方不在线</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeExpired</t>
+          <t>MatchChallengeTargetBusy</t>
         </is>
       </c>
       <c r="B221" s="0" t="inlineStr">
         <is>
-          <t>挑战已过期</t>
+          <t>对方正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeNotTarget</t>
+          <t>MatchChallengeSelfBusy</t>
         </is>
       </c>
       <c r="B222" s="0" t="inlineStr">
         <is>
-          <t>你不是该挑战的对象</t>
+          <t>你正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateWhileQueued</t>
+          <t>MatchChallengePending</t>
         </is>
       </c>
       <c r="B223" s="0" t="inlineStr">
         <is>
-          <t>匹配中无法观战</t>
+          <t>已有待应答的挑战</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateWhileInBattle</t>
+          <t>MatchChallengeExpired</t>
         </is>
       </c>
       <c r="B224" s="0" t="inlineStr">
         <is>
-          <t>战斗中无法观战</t>
+          <t>挑战已过期</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t>MatchAlreadyWatching</t>
+          <t>MatchChallengeNotTarget</t>
         </is>
       </c>
       <c r="B225" s="0" t="inlineStr">
         <is>
-          <t>已在观战中</t>
+          <t>你不是该挑战的对象</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t>MatchNoWatchableBattle</t>
+          <t>MatchSpectateWhileQueued</t>
         </is>
       </c>
       <c r="B226" s="0" t="inlineStr">
         <is>
-          <t>当前没有可观战的战斗</t>
+          <t>匹配中无法观战</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t>MatchBattleNotWatchable</t>
+          <t>MatchSpectateWhileInBattle</t>
         </is>
       </c>
       <c r="B227" s="0" t="inlineStr">
         <is>
-          <t>该战斗无法观战</t>
+          <t>战斗中无法观战</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateOffline</t>
+          <t>MatchAlreadyWatching</t>
         </is>
       </c>
       <c r="B228" s="0" t="inlineStr">
         <is>
-          <t>观战会话已断开</t>
+          <t>已在观战中</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t>MatchNotInScene</t>
+          <t>MatchNoWatchableBattle</t>
         </is>
       </c>
       <c r="B229" s="0" t="inlineStr">
         <is>
-          <t>请先进入场景</t>
+          <t>当前没有可观战的战斗</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t>// 以下号段为移植域预留，建组时把本行改成组头即可：</t>
+          <t>MatchBattleNotWatchable</t>
+        </is>
+      </c>
+      <c r="B230" s="0" t="inlineStr">
+        <is>
+          <t>该战斗无法观战</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t>//   mail_error 17000 / chat_error 18000 / auction_error 19000</t>
+          <t>MatchSpectateOffline</t>
+        </is>
+      </c>
+      <c r="B231" s="0" t="inlineStr">
+        <is>
+          <t>观战会话已断开</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t>//   rank_error 21000 / dialogue_error 22000 / battle_result_error 23000 / grant_error 24000</t>
-        </is>
-      </c>
-    </row>
-    <row r="233"/>
+          <t>MatchNotInScene</t>
+        </is>
+      </c>
+      <c r="B232" s="0" t="inlineStr">
+        <is>
+          <t>请先进入场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="0" t="inlineStr">
+        <is>
+          <t>// 以下号段为移植域预留，建组时把本行改成组头即可：</t>
+        </is>
+      </c>
+    </row>
     <row r="234">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t>//trade_error base=20000 width=1000</t>
+          <t>//   mail_error 17000 / chat_error 18000 / auction_error 19000</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t>TradeListingNotFound</t>
-        </is>
-      </c>
-      <c r="B235" s="0" t="inlineStr">
-        <is>
-          <t>商品不存在或已下架</t>
-        </is>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" s="0" t="inlineStr">
-        <is>
-          <t>TradeHomeZoneUnknown</t>
-        </is>
-      </c>
-      <c r="B236" s="0" t="inlineStr">
-        <is>
-          <t>角色归属区服未确认，暂时无法使用聚宝斋</t>
-        </is>
-      </c>
-    </row>
+          <t>//   rank_error 21000 / dialogue_error 22000 / battle_result_error 23000 / grant_error 24000</t>
+        </is>
+      </c>
+    </row>
+    <row r="236"/>
     <row r="237">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t>TradeFavoriteLimitReached</t>
-        </is>
-      </c>
-      <c r="B237" s="0" t="inlineStr">
-        <is>
-          <t>收藏数量已达上限，请先取消部分收藏</t>
+          <t>//trade_error base=20000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t>TradeFeatureDisabled</t>
+          <t>TradeListingNotFound</t>
         </is>
       </c>
       <c r="B238" s="0" t="inlineStr">
         <is>
-          <t>该功能尚未开放</t>
-        </is>
-      </c>
-    </row>
-    <row r="239"/>
+          <t>商品不存在或已下架</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="0" t="inlineStr">
+        <is>
+          <t>TradeHomeZoneUnknown</t>
+        </is>
+      </c>
+      <c r="B239" s="0" t="inlineStr">
+        <is>
+          <t>角色归属区服未确认，暂时无法使用聚宝斋</t>
+        </is>
+      </c>
+    </row>
     <row r="240">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t>//attribute_error base=25000 width=1000</t>
+          <t>TradeFavoriteLimitReached</t>
+        </is>
+      </c>
+      <c r="B240" s="0" t="inlineStr">
+        <is>
+          <t>收藏数量已达上限，请先取消部分收藏</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t>AttributePoolNotFound</t>
+          <t>TradeFeatureDisabled</t>
         </is>
       </c>
       <c r="B241" s="0" t="inlineStr">
         <is>
-          <t>属性池不存在</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" s="0" t="inlineStr">
-        <is>
-          <t>AttributePoolLocked</t>
-        </is>
-      </c>
-      <c r="B242" s="0" t="inlineStr">
-        <is>
-          <t>该属性池尚未解锁</t>
-        </is>
-      </c>
-    </row>
+          <t>该功能尚未开放</t>
+        </is>
+      </c>
+    </row>
+    <row r="242"/>
     <row r="243">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t>AttributeDimensionNotFound</t>
-        </is>
-      </c>
-      <c r="B243" s="0" t="inlineStr">
-        <is>
-          <t>属性维度不存在</t>
+          <t>//attribute_error base=25000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t>AttributePointsNotEnough</t>
+          <t>AttributePoolNotFound</t>
         </is>
       </c>
       <c r="B244" s="0" t="inlineStr">
         <is>
-          <t>剩余点数不足</t>
+          <t>属性池不存在</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t>AttributePointsCannotDecrease</t>
+          <t>AttributePoolLocked</t>
         </is>
       </c>
       <c r="B245" s="0" t="inlineStr">
         <is>
-          <t>已分配的点数不能减少,请使用重置</t>
+          <t>该属性池尚未解锁</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t>AttributeDimensionCapExceeded</t>
+          <t>AttributeDimensionNotFound</t>
         </is>
       </c>
       <c r="B246" s="0" t="inlineStr">
         <is>
-          <t>超过单项可分配上限</t>
+          <t>属性维度不存在</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeNotFound</t>
+          <t>AttributePointsNotEnough</t>
         </is>
       </c>
       <c r="B247" s="0" t="inlineStr">
         <is>
-          <t>加点方案不存在</t>
+          <t>剩余点数不足</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeLimitReached</t>
+          <t>AttributePointsCannotDecrease</t>
         </is>
       </c>
       <c r="B248" s="0" t="inlineStr">
         <is>
-          <t>加点方案数量已达上限</t>
+          <t>已分配的点数不能减少,请使用重置</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeSwitchCooldown</t>
+          <t>AttributeDimensionCapExceeded</t>
         </is>
       </c>
       <c r="B249" s="0" t="inlineStr">
         <is>
-          <t>方案切换冷却中</t>
+          <t>超过单项可分配上限</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeNameInvalid</t>
+          <t>AttributeSchemeNotFound</t>
         </is>
       </c>
       <c r="B250" s="0" t="inlineStr">
         <is>
-          <t>方案名称不合法</t>
+          <t>加点方案不存在</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeAlreadyActive</t>
+          <t>AttributeSchemeLimitReached</t>
         </is>
       </c>
       <c r="B251" s="0" t="inlineStr">
         <is>
-          <t>已经是当前方案</t>
+          <t>加点方案数量已达上限</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="0" t="inlineStr">
         <is>
-          <t>AttributeInBattle</t>
+          <t>AttributeSchemeSwitchCooldown</t>
         </is>
       </c>
       <c r="B252" s="0" t="inlineStr">
         <is>
-          <t>战斗中不能修改属性</t>
+          <t>方案切换冷却中</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t>AttributeGoldNotEnough</t>
+          <t>AttributeSchemeNameInvalid</t>
         </is>
       </c>
       <c r="B253" s="0" t="inlineStr">
         <is>
-          <t>金币不足</t>
+          <t>方案名称不合法</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t>AttributeNoAutoPlan</t>
+          <t>AttributeSchemeAlreadyActive</t>
         </is>
       </c>
       <c r="B254" s="0" t="inlineStr">
         <is>
-          <t>没有可用的自动加点方案</t>
+          <t>已经是当前方案</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t>AttributeNothingToChange</t>
+          <t>AttributeInBattle</t>
         </is>
       </c>
       <c r="B255" s="0" t="inlineStr">
         <is>
-          <t>属性没有变化</t>
-        </is>
-      </c>
-    </row>
-    <row r="256"/>
+          <t>战斗中不能修改属性</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="0" t="inlineStr">
+        <is>
+          <t>AttributeGoldNotEnough</t>
+        </is>
+      </c>
+      <c r="B256" s="0" t="inlineStr">
+        <is>
+          <t>金币不足</t>
+        </is>
+      </c>
+    </row>
     <row r="257">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t>//pet_error base=26000 width=1000</t>
+          <t>AttributeNoAutoPlan</t>
+        </is>
+      </c>
+      <c r="B257" s="0" t="inlineStr">
+        <is>
+          <t>没有可用的自动加点方案</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t>PetNotFound</t>
+          <t>AttributeNothingToChange</t>
         </is>
       </c>
       <c r="B258" s="0" t="inlineStr">
         <is>
-          <t>宝宝不存在</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" s="0" t="inlineStr">
-        <is>
-          <t>PetTableRowMissing</t>
-        </is>
-      </c>
-      <c r="B259" s="0" t="inlineStr">
-        <is>
-          <t>宝宝数据已失效,请联系客服</t>
-        </is>
-      </c>
-    </row>
+          <t>属性没有变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="259"/>
     <row r="260">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t>PetSlotFull</t>
-        </is>
-      </c>
-      <c r="B260" s="0" t="inlineStr">
-        <is>
-          <t>可携带的宝宝数量已达上限</t>
+          <t>//pet_error base=26000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t>PetOwnerLevelNotEnough</t>
+          <t>PetNotFound</t>
         </is>
       </c>
       <c r="B261" s="0" t="inlineStr">
         <is>
-          <t>主人等级不足,还不能携带这只宝宝</t>
+          <t>宝宝不存在</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="0" t="inlineStr">
         <is>
-          <t>PetAlreadyActive</t>
+          <t>PetTableRowMissing</t>
         </is>
       </c>
       <c r="B262" s="0" t="inlineStr">
         <is>
-          <t>这只宝宝已经在出战中</t>
+          <t>宝宝数据已失效,请联系客服</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t>PetNotActive</t>
+          <t>PetSlotFull</t>
         </is>
       </c>
       <c r="B263" s="0" t="inlineStr">
         <is>
-          <t>当前没有出战的宝宝</t>
+          <t>可携带的宝宝数量已达上限</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t>PetSummonCooldown</t>
+          <t>PetOwnerLevelNotEnough</t>
         </is>
       </c>
       <c r="B264" s="0" t="inlineStr">
         <is>
-          <t>操作太频繁,请稍后再试</t>
+          <t>主人等级不足,还不能携带这只宝宝</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t>PetNameInvalid</t>
+          <t>PetAlreadyActive</t>
         </is>
       </c>
       <c r="B265" s="0" t="inlineStr">
         <is>
-          <t>宝宝名称不合法</t>
+          <t>这只宝宝已经在出战中</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t>PetInBattle</t>
+          <t>PetNotActive</t>
         </is>
       </c>
       <c r="B266" s="0" t="inlineStr">
         <is>
-          <t>战斗中不能操作宝宝</t>
+          <t>当前没有出战的宝宝</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t>PetPointsNotEnough</t>
+          <t>PetSummonCooldown</t>
         </is>
       </c>
       <c r="B267" s="0" t="inlineStr">
         <is>
-          <t>宝宝剩余点数不足</t>
+          <t>操作太频繁,请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t>PetPointsCannotDecrease</t>
+          <t>PetNameInvalid</t>
         </is>
       </c>
       <c r="B268" s="0" t="inlineStr">
         <is>
-          <t>已分配的点数不能减少,请使用洗点</t>
+          <t>宝宝名称不合法</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="0" t="inlineStr">
         <is>
-          <t>PetDimensionCapExceeded</t>
+          <t>PetInBattle</t>
         </is>
       </c>
       <c r="B269" s="0" t="inlineStr">
         <is>
-          <t>超过单项可分配上限</t>
+          <t>战斗中不能操作宝宝</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t>PetDimensionNotFound</t>
+          <t>PetPointsNotEnough</t>
         </is>
       </c>
       <c r="B270" s="0" t="inlineStr">
         <is>
-          <t>宝宝属性维度不存在</t>
+          <t>宝宝剩余点数不足</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="0" t="inlineStr">
         <is>
-          <t>PetGoldNotEnough</t>
+          <t>PetPointsCannotDecrease</t>
         </is>
       </c>
       <c r="B271" s="0" t="inlineStr">
         <is>
-          <t>金币不足</t>
+          <t>已分配的点数不能减少,请使用洗点</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="0" t="inlineStr">
         <is>
-          <t>PetNoAutoPlan</t>
+          <t>PetDimensionCapExceeded</t>
         </is>
       </c>
       <c r="B272" s="0" t="inlineStr">
         <is>
-          <t>没有可用的自动加点方案</t>
+          <t>超过单项可分配上限</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="0" t="inlineStr">
         <is>
-          <t>PetNothingToChange</t>
+          <t>PetDimensionNotFound</t>
         </is>
       </c>
       <c r="B273" s="0" t="inlineStr">
         <is>
-          <t>宝宝属性没有变化</t>
+          <t>宝宝属性维度不存在</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="0" t="inlineStr">
         <is>
+          <t>PetGoldNotEnough</t>
+        </is>
+      </c>
+      <c r="B274" s="0" t="inlineStr">
+        <is>
+          <t>金币不足</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="0" t="inlineStr">
+        <is>
+          <t>PetNoAutoPlan</t>
+        </is>
+      </c>
+      <c r="B275" s="0" t="inlineStr">
+        <is>
+          <t>没有可用的自动加点方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="0" t="inlineStr">
+        <is>
+          <t>PetNothingToChange</t>
+        </is>
+      </c>
+      <c r="B276" s="0" t="inlineStr">
+        <is>
+          <t>宝宝属性没有变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="0" t="inlineStr">
+        <is>
           <t>PetIdGenerateFailed</t>
         </is>
       </c>
-      <c r="B274" s="0" t="inlineStr">
+      <c r="B277" s="0" t="inlineStr">
         <is>
           <t>宝宝创建失败,请稍后再试</t>
         </is>
       </c>
-      <c r="C274" s="0" t="n">
+      <c r="C277" s="0" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
+    <row r="278"/>
+    <row r="279">
+      <c r="A279" s="0" t="inlineStr">
         <is>
           <t>//asset_error base=27000 width=1000</t>
         </is>
       </c>
     </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
+    <row r="280">
+      <c r="A280" s="0" t="inlineStr">
         <is>
           <t>AssetCurrencyInsufficient</t>
         </is>
       </c>
-      <c r="B277" t="inlineStr">
+      <c r="B280" s="0" t="inlineStr">
         <is>
           <t>货币不足</t>
         </is>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
+    <row r="281">
+      <c r="A281" s="0" t="inlineStr">
         <is>
           <t>AssetBagFull</t>
         </is>
       </c>
-      <c r="B278" t="inlineStr">
+      <c r="B281" s="0" t="inlineStr">
         <is>
           <t>背包已满，请腾出空间，之后会重试发放；超过时限可能取消</t>
         </is>
       </c>
     </row>
-    <row r="279">
-      <c r="A279" t="inlineStr">
+    <row r="282">
+      <c r="A282" s="0" t="inlineStr">
         <is>
           <t>AssetInBattle</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr">
+      <c r="B282" s="0" t="inlineStr">
         <is>
           <t>战斗中暂不结算，稍后自动重试；超过时限可能取消</t>
         </is>
       </c>
     </row>
-    <row r="280">
-      <c r="A280" t="inlineStr">
+    <row r="283">
+      <c r="A283" s="0" t="inlineStr">
         <is>
           <t>AssetFrozen</t>
         </is>
       </c>
-      <c r="B280" t="inlineStr">
+      <c r="B283" s="0" t="inlineStr">
         <is>
           <t>角色迁移中，稍后自动重试；超过时限可能取消</t>
         </is>
       </c>
     </row>
-    <row r="281">
-      <c r="A281" t="inlineStr">
+    <row r="284">
+      <c r="A284" s="0" t="inlineStr">
         <is>
           <t>AssetInvalidBundle</t>
         </is>
       </c>
-      <c r="B281" t="inlineStr">
+      <c r="B284" s="0" t="inlineStr">
         <is>
           <t>资产指令无效</t>
         </is>
       </c>
-      <c r="C281" t="n">
+      <c r="C284" s="0" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="282">
-      <c r="A282" t="inlineStr">
+    <row r="285">
+      <c r="A285" s="0" t="inlineStr">
         <is>
           <t>AssetBlocked</t>
         </is>
       </c>
-      <c r="B282" t="inlineStr">
+      <c r="B285" s="0" t="inlineStr">
         <is>
           <t>该资产当前被禁止获取</t>
         </is>
       </c>
     </row>
-    <row r="283">
-      <c r="A283" t="inlineStr">
+    <row r="286">
+      <c r="A286" s="0" t="inlineStr">
         <is>
           <t>AssetPlayerNotHere</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr">
+      <c r="B286" s="0" t="inlineStr">
         <is>
           <t>角色不在线，上线后重试；超过时限可能取消</t>
         </is>
       </c>
     </row>
-    <row r="284">
-      <c r="A284" t="inlineStr">
+    <row r="287">
+      <c r="A287" s="0" t="inlineStr">
         <is>
           <t>AssetPartialApplied</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr">
+      <c r="B287" s="0" t="inlineStr">
         <is>
           <t>资产只发放了一部分，已记录，将由客服补偿</t>
         </is>
       </c>
-      <c r="C284" t="n">
+      <c r="C287" s="0" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="285">
-      <c r="A285" t="inlineStr">
+    <row r="288">
+      <c r="A288" s="0" t="inlineStr">
         <is>
           <t>AssetAuthFailed</t>
         </is>
       </c>
-      <c r="B285" t="inlineStr">
+      <c r="B288" s="0" t="inlineStr">
         <is>
           <t>资产指令校验失败</t>
         </is>
       </c>
-      <c r="C285" t="n">
+      <c r="C288" s="0" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP：保存全部进度 2026-09-20 22:55 -04:00（好友系统 go/friend 与 robot handlers、GuildDonate/GuildShop/RoleNameRule 配置表、guild phase2/leaderboard 文档）
</commit_message>
<xml_diff>
--- a/data/tip/Tip.xlsx
+++ b/data/tip/Tip.xlsx
@@ -1020,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C291"/>
+  <dimension ref="A1:C301"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="8" customWidth="1" style="2" min="3" max="3"/>
@@ -1060,6 +1060,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
@@ -1077,6 +1078,19 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
@@ -3098,262 +3112,261 @@
     <row r="203">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>//friend_error base=15000 width=1000</t>
+          <t>GuildFundsInsufficient</t>
+        </is>
+      </c>
+      <c r="B203" s="0" t="inlineStr">
+        <is>
+          <t>帮会资金不足</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t>FriendCannotAddSelf</t>
+          <t>GuildMaxLevel</t>
         </is>
       </c>
       <c r="B204" s="0" t="inlineStr">
         <is>
-          <t>不能添加自己为好友</t>
+          <t>帮会已达最高等级</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t>FriendAlreadyFriends</t>
+          <t>GuildDonateLimit</t>
         </is>
       </c>
       <c r="B205" s="0" t="inlineStr">
         <is>
-          <t>你们已经是好友了</t>
+          <t>今日该项捐献次数已用完</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t>FriendListFull</t>
+          <t>GuildCurrencyInsufficient</t>
         </is>
       </c>
       <c r="B206" s="0" t="inlineStr">
         <is>
-          <t>好友列表已满</t>
+          <t>货币不足，无法捐献</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t>FriendRequestAlreadySent</t>
+          <t>GuildAssetPending</t>
         </is>
       </c>
       <c r="B207" s="0" t="inlineStr">
         <is>
-          <t>已发送过好友申请</t>
+          <t>有未结算的帮会资产操作，请稍后再试</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t>FriendTargetListFull</t>
+          <t>GuildAssetRejected</t>
         </is>
       </c>
       <c r="B208" s="0" t="inlineStr">
         <is>
-          <t>对方好友列表已满</t>
+          <t>资产结算失败，本次操作已撤销</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t>FriendNoPendingRequest</t>
+          <t>GuildShopGoodsNotFound</t>
         </is>
       </c>
       <c r="B209" s="0" t="inlineStr">
         <is>
-          <t>没有待处理的好友申请</t>
+          <t>兑换商品不存在</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t>FriendTooManyPending</t>
+          <t>GuildShopLevelTooLow</t>
         </is>
       </c>
       <c r="B210" s="0" t="inlineStr">
         <is>
-          <t>待处理的申请过多</t>
+          <t>帮会等级不足</t>
         </is>
       </c>
     </row>
     <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>FriendBlocked</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>对方已将你拉黑</t>
+      <c r="A211" s="0" t="inlineStr">
+        <is>
+          <t>GuildShopLimit</t>
+        </is>
+      </c>
+      <c r="B211" s="0" t="inlineStr">
+        <is>
+          <t>已达限购数量</t>
         </is>
       </c>
     </row>
     <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>FriendBlockListFull</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>黑名单已满</t>
+      <c r="A212" s="0" t="inlineStr">
+        <is>
+          <t>GuildContributionInsufficient</t>
+        </is>
+      </c>
+      <c r="B212" s="0" t="inlineStr">
+        <is>
+          <t>可用帮贡不足</t>
         </is>
       </c>
     </row>
     <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>FriendTargetInboxFull</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>对方的好友申请已满</t>
+      <c r="A213" s="0" t="inlineStr">
+        <is>
+          <t>//friend_error base=15000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t>//match_error base=16000 width=1000</t>
+          <t>FriendCannotAddSelf</t>
+        </is>
+      </c>
+      <c r="B214" s="0" t="inlineStr">
+        <is>
+          <t>不能添加自己为好友</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t>MatchInBattle</t>
+          <t>FriendAlreadyFriends</t>
         </is>
       </c>
       <c r="B215" s="0" t="inlineStr">
         <is>
-          <t>你正在战斗中</t>
+          <t>你们已经是好友了</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t>MatchAlreadyQueued</t>
+          <t>FriendListFull</t>
         </is>
       </c>
       <c r="B216" s="0" t="inlineStr">
         <is>
-          <t>已在匹配队列中</t>
+          <t>好友列表已满</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t>MatchModeNotOpen</t>
+          <t>FriendRequestAlreadySent</t>
         </is>
       </c>
       <c r="B217" s="0" t="inlineStr">
         <is>
-          <t>该匹配模式暂未开放</t>
+          <t>已发送过好友申请</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t>MatchTeamSizeNotConfigured</t>
+          <t>FriendTargetListFull</t>
         </is>
       </c>
       <c r="B218" s="0" t="inlineStr">
         <is>
-          <t>队伍人数未配置</t>
+          <t>对方好友列表已满</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t>MatchInternal</t>
+          <t>FriendNoPendingRequest</t>
         </is>
       </c>
       <c r="B219" s="0" t="inlineStr">
         <is>
-          <t>服务繁忙，请稍后重试</t>
-        </is>
-      </c>
-      <c r="C219" s="0" t="n"/>
+          <t>没有待处理的好友申请</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t>MatchTicketMismatch</t>
+          <t>FriendTooManyPending</t>
         </is>
       </c>
       <c r="B220" s="0" t="inlineStr">
         <is>
-          <t>匹配凭据不匹配</t>
+          <t>待处理的申请过多</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t>MatchCancelTooLate</t>
+          <t>FriendBlocked</t>
         </is>
       </c>
       <c r="B221" s="0" t="inlineStr">
         <is>
-          <t>匹配已开始，无法取消</t>
+          <t>无法添加该玩家为好友</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeSelf</t>
+          <t>FriendBlockListFull</t>
         </is>
       </c>
       <c r="B222" s="0" t="inlineStr">
         <is>
-          <t>不能挑战自己</t>
+          <t>黑名单已满</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeTargetOffline</t>
+          <t>FriendTargetInboxFull</t>
         </is>
       </c>
       <c r="B223" s="0" t="inlineStr">
         <is>
-          <t>对方不在线</t>
+          <t>对方的好友申请已满</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeTargetBusy</t>
-        </is>
-      </c>
-      <c r="B224" s="0" t="inlineStr">
-        <is>
-          <t>对方正在战斗中</t>
+          <t>//match_error base=16000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeSelfBusy</t>
+          <t>MatchInBattle</t>
         </is>
       </c>
       <c r="B225" s="0" t="inlineStr">
@@ -3365,725 +3378,846 @@
     <row r="226">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengePending</t>
+          <t>MatchAlreadyQueued</t>
         </is>
       </c>
       <c r="B226" s="0" t="inlineStr">
         <is>
-          <t>已有待应答的挑战</t>
+          <t>已在匹配队列中</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeExpired</t>
+          <t>MatchModeNotOpen</t>
         </is>
       </c>
       <c r="B227" s="0" t="inlineStr">
         <is>
-          <t>挑战已过期</t>
+          <t>该匹配模式暂未开放</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t>MatchChallengeNotTarget</t>
+          <t>MatchTeamSizeNotConfigured</t>
         </is>
       </c>
       <c r="B228" s="0" t="inlineStr">
         <is>
-          <t>你不是该挑战的对象</t>
+          <t>队伍人数未配置</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateWhileQueued</t>
+          <t>MatchInternal</t>
         </is>
       </c>
       <c r="B229" s="0" t="inlineStr">
         <is>
-          <t>匹配中无法观战</t>
-        </is>
-      </c>
+          <t>服务繁忙，请稍后重试</t>
+        </is>
+      </c>
+      <c r="C229" s="0" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateWhileInBattle</t>
+          <t>MatchTicketMismatch</t>
         </is>
       </c>
       <c r="B230" s="0" t="inlineStr">
         <is>
-          <t>战斗中无法观战</t>
+          <t>匹配凭据不匹配</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t>MatchAlreadyWatching</t>
+          <t>MatchCancelTooLate</t>
         </is>
       </c>
       <c r="B231" s="0" t="inlineStr">
         <is>
-          <t>已在观战中</t>
+          <t>匹配已开始，无法取消</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t>MatchNoWatchableBattle</t>
+          <t>MatchChallengeSelf</t>
         </is>
       </c>
       <c r="B232" s="0" t="inlineStr">
         <is>
-          <t>当前没有可观战的战斗</t>
+          <t>不能挑战自己</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t>MatchBattleNotWatchable</t>
+          <t>MatchChallengeTargetOffline</t>
         </is>
       </c>
       <c r="B233" s="0" t="inlineStr">
         <is>
-          <t>该战斗无法观战</t>
+          <t>对方不在线</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t>MatchSpectateOffline</t>
+          <t>MatchChallengeTargetBusy</t>
         </is>
       </c>
       <c r="B234" s="0" t="inlineStr">
         <is>
-          <t>观战会话已断开</t>
+          <t>对方正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t>MatchNotInScene</t>
+          <t>MatchChallengeSelfBusy</t>
         </is>
       </c>
       <c r="B235" s="0" t="inlineStr">
         <is>
-          <t>请先进入场景</t>
+          <t>你正在战斗中</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t>// 以下号段为移植域预留，建组时把本行改成组头即可：</t>
+          <t>MatchChallengePending</t>
+        </is>
+      </c>
+      <c r="B236" s="0" t="inlineStr">
+        <is>
+          <t>已有待应答的挑战</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t>//   mail_error 17000 / chat_error 18000 / auction_error 19000</t>
+          <t>MatchChallengeExpired</t>
+        </is>
+      </c>
+      <c r="B237" s="0" t="inlineStr">
+        <is>
+          <t>挑战已过期</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t>//   rank_error 21000 / dialogue_error 22000 / battle_result_error 23000 / grant_error 24000</t>
-        </is>
-      </c>
-    </row>
-    <row r="239"/>
+          <t>MatchChallengeNotTarget</t>
+        </is>
+      </c>
+      <c r="B238" s="0" t="inlineStr">
+        <is>
+          <t>你不是该挑战的对象</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="0" t="inlineStr">
+        <is>
+          <t>MatchSpectateWhileQueued</t>
+        </is>
+      </c>
+      <c r="B239" s="0" t="inlineStr">
+        <is>
+          <t>匹配中无法观战</t>
+        </is>
+      </c>
+    </row>
     <row r="240">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t>//trade_error base=20000 width=1000</t>
+          <t>MatchSpectateWhileInBattle</t>
+        </is>
+      </c>
+      <c r="B240" s="0" t="inlineStr">
+        <is>
+          <t>战斗中无法观战</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t>TradeListingNotFound</t>
+          <t>MatchAlreadyWatching</t>
         </is>
       </c>
       <c r="B241" s="0" t="inlineStr">
         <is>
-          <t>商品不存在或已下架</t>
+          <t>已在观战中</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t>TradeHomeZoneUnknown</t>
+          <t>MatchNoWatchableBattle</t>
         </is>
       </c>
       <c r="B242" s="0" t="inlineStr">
         <is>
-          <t>角色归属区服未确认，暂时无法使用聚宝斋</t>
+          <t>当前没有可观战的战斗</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t>TradeFavoriteLimitReached</t>
+          <t>MatchBattleNotWatchable</t>
         </is>
       </c>
       <c r="B243" s="0" t="inlineStr">
         <is>
-          <t>收藏数量已达上限，请先取消部分收藏</t>
+          <t>该战斗无法观战</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t>TradeFeatureDisabled</t>
+          <t>MatchSpectateOffline</t>
         </is>
       </c>
       <c r="B244" s="0" t="inlineStr">
         <is>
-          <t>该功能尚未开放</t>
-        </is>
-      </c>
-    </row>
-    <row r="245"/>
+          <t>观战会话已断开</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="0" t="inlineStr">
+        <is>
+          <t>MatchNotInScene</t>
+        </is>
+      </c>
+      <c r="B245" s="0" t="inlineStr">
+        <is>
+          <t>请先进入场景</t>
+        </is>
+      </c>
+    </row>
     <row r="246">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t>//attribute_error base=25000 width=1000</t>
+          <t>// 以下号段为移植域预留，建组时把本行改成组头即可：</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t>AttributePoolNotFound</t>
-        </is>
-      </c>
-      <c r="B247" s="0" t="inlineStr">
-        <is>
-          <t>属性池不存在</t>
+          <t>//   mail_error 17000 / chat_error 18000 / auction_error 19000</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t>AttributePoolLocked</t>
-        </is>
-      </c>
-      <c r="B248" s="0" t="inlineStr">
-        <is>
-          <t>该属性池尚未解锁</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" s="0" t="inlineStr">
-        <is>
-          <t>AttributeDimensionNotFound</t>
-        </is>
-      </c>
-      <c r="B249" s="0" t="inlineStr">
-        <is>
-          <t>属性维度不存在</t>
-        </is>
-      </c>
-    </row>
+          <t>//   rank_error 21000 / dialogue_error 22000 / battle_result_error 23000 / grant_error 24000</t>
+        </is>
+      </c>
+    </row>
+    <row r="249"/>
     <row r="250">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t>AttributePointsNotEnough</t>
-        </is>
-      </c>
-      <c r="B250" s="0" t="inlineStr">
-        <is>
-          <t>剩余点数不足</t>
+          <t>//trade_error base=20000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t>AttributePointsCannotDecrease</t>
+          <t>TradeListingNotFound</t>
         </is>
       </c>
       <c r="B251" s="0" t="inlineStr">
         <is>
-          <t>已分配的点数不能减少,请使用重置</t>
+          <t>商品不存在或已下架</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="0" t="inlineStr">
         <is>
-          <t>AttributeDimensionCapExceeded</t>
+          <t>TradeHomeZoneUnknown</t>
         </is>
       </c>
       <c r="B252" s="0" t="inlineStr">
         <is>
-          <t>超过单项可分配上限</t>
+          <t>角色归属区服未确认，暂时无法使用聚宝斋</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeNotFound</t>
+          <t>TradeFavoriteLimitReached</t>
         </is>
       </c>
       <c r="B253" s="0" t="inlineStr">
         <is>
-          <t>加点方案不存在</t>
+          <t>收藏数量已达上限，请先取消部分收藏</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeLimitReached</t>
+          <t>TradeFeatureDisabled</t>
         </is>
       </c>
       <c r="B254" s="0" t="inlineStr">
         <is>
-          <t>加点方案数量已达上限</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="0" t="inlineStr">
-        <is>
-          <t>AttributeSchemeSwitchCooldown</t>
-        </is>
-      </c>
-      <c r="B255" s="0" t="inlineStr">
-        <is>
-          <t>方案切换冷却中</t>
-        </is>
-      </c>
-    </row>
+          <t>该功能尚未开放</t>
+        </is>
+      </c>
+    </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeNameInvalid</t>
-        </is>
-      </c>
-      <c r="B256" s="0" t="inlineStr">
-        <is>
-          <t>方案名称不合法</t>
+          <t>//attribute_error base=25000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t>AttributeSchemeAlreadyActive</t>
+          <t>AttributePoolNotFound</t>
         </is>
       </c>
       <c r="B257" s="0" t="inlineStr">
         <is>
-          <t>已经是当前方案</t>
+          <t>属性池不存在</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t>AttributeInBattle</t>
+          <t>AttributePoolLocked</t>
         </is>
       </c>
       <c r="B258" s="0" t="inlineStr">
         <is>
-          <t>战斗中不能修改属性</t>
+          <t>该属性池尚未解锁</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="0" t="inlineStr">
         <is>
-          <t>AttributeGoldNotEnough</t>
+          <t>AttributeDimensionNotFound</t>
         </is>
       </c>
       <c r="B259" s="0" t="inlineStr">
         <is>
-          <t>金币不足</t>
+          <t>属性维度不存在</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t>AttributeNoAutoPlan</t>
+          <t>AttributePointsNotEnough</t>
         </is>
       </c>
       <c r="B260" s="0" t="inlineStr">
         <is>
-          <t>没有可用的自动加点方案</t>
+          <t>剩余点数不足</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t>AttributeNothingToChange</t>
+          <t>AttributePointsCannotDecrease</t>
         </is>
       </c>
       <c r="B261" s="0" t="inlineStr">
         <is>
-          <t>属性没有变化</t>
-        </is>
-      </c>
-    </row>
-    <row r="262"/>
+          <t>已分配的点数不能减少,请使用重置</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="0" t="inlineStr">
+        <is>
+          <t>AttributeDimensionCapExceeded</t>
+        </is>
+      </c>
+      <c r="B262" s="0" t="inlineStr">
+        <is>
+          <t>超过单项可分配上限</t>
+        </is>
+      </c>
+    </row>
     <row r="263">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t>//pet_error base=26000 width=1000</t>
+          <t>AttributeSchemeNotFound</t>
+        </is>
+      </c>
+      <c r="B263" s="0" t="inlineStr">
+        <is>
+          <t>加点方案不存在</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t>PetNotFound</t>
+          <t>AttributeSchemeLimitReached</t>
         </is>
       </c>
       <c r="B264" s="0" t="inlineStr">
         <is>
-          <t>宝宝不存在</t>
+          <t>加点方案数量已达上限</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t>PetTableRowMissing</t>
+          <t>AttributeSchemeSwitchCooldown</t>
         </is>
       </c>
       <c r="B265" s="0" t="inlineStr">
         <is>
-          <t>宝宝数据已失效,请联系客服</t>
+          <t>方案切换冷却中</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t>PetSlotFull</t>
+          <t>AttributeSchemeNameInvalid</t>
         </is>
       </c>
       <c r="B266" s="0" t="inlineStr">
         <is>
-          <t>可携带的宝宝数量已达上限</t>
+          <t>方案名称不合法</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t>PetOwnerLevelNotEnough</t>
+          <t>AttributeSchemeAlreadyActive</t>
         </is>
       </c>
       <c r="B267" s="0" t="inlineStr">
         <is>
-          <t>主人等级不足,还不能携带这只宝宝</t>
+          <t>已经是当前方案</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t>PetAlreadyActive</t>
+          <t>AttributeInBattle</t>
         </is>
       </c>
       <c r="B268" s="0" t="inlineStr">
         <is>
-          <t>这只宝宝已经在出战中</t>
+          <t>战斗中不能修改属性</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="0" t="inlineStr">
         <is>
-          <t>PetNotActive</t>
+          <t>AttributeGoldNotEnough</t>
         </is>
       </c>
       <c r="B269" s="0" t="inlineStr">
         <is>
-          <t>当前没有出战的宝宝</t>
+          <t>金币不足</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t>PetSummonCooldown</t>
+          <t>AttributeNoAutoPlan</t>
         </is>
       </c>
       <c r="B270" s="0" t="inlineStr">
         <is>
-          <t>操作太频繁,请稍后再试</t>
+          <t>没有可用的自动加点方案</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="0" t="inlineStr">
         <is>
-          <t>PetNameInvalid</t>
+          <t>AttributeNothingToChange</t>
         </is>
       </c>
       <c r="B271" s="0" t="inlineStr">
         <is>
-          <t>宝宝名称不合法</t>
-        </is>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" s="0" t="inlineStr">
-        <is>
-          <t>PetInBattle</t>
-        </is>
-      </c>
-      <c r="B272" s="0" t="inlineStr">
-        <is>
-          <t>战斗中不能操作宝宝</t>
-        </is>
-      </c>
-    </row>
+          <t>属性没有变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="272"/>
     <row r="273">
       <c r="A273" s="0" t="inlineStr">
         <is>
-          <t>PetPointsNotEnough</t>
-        </is>
-      </c>
-      <c r="B273" s="0" t="inlineStr">
-        <is>
-          <t>宝宝剩余点数不足</t>
+          <t>//pet_error base=26000 width=1000</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="0" t="inlineStr">
         <is>
-          <t>PetPointsCannotDecrease</t>
+          <t>PetNotFound</t>
         </is>
       </c>
       <c r="B274" s="0" t="inlineStr">
         <is>
-          <t>已分配的点数不能减少,请使用洗点</t>
+          <t>宝宝不存在</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="0" t="inlineStr">
         <is>
-          <t>PetDimensionCapExceeded</t>
+          <t>PetTableRowMissing</t>
         </is>
       </c>
       <c r="B275" s="0" t="inlineStr">
         <is>
-          <t>超过单项可分配上限</t>
+          <t>宝宝数据已失效,请联系客服</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="0" t="inlineStr">
         <is>
-          <t>PetDimensionNotFound</t>
+          <t>PetSlotFull</t>
         </is>
       </c>
       <c r="B276" s="0" t="inlineStr">
         <is>
-          <t>宝宝属性维度不存在</t>
+          <t>可携带的宝宝数量已达上限</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="0" t="inlineStr">
         <is>
-          <t>PetGoldNotEnough</t>
+          <t>PetOwnerLevelNotEnough</t>
         </is>
       </c>
       <c r="B277" s="0" t="inlineStr">
         <is>
-          <t>金币不足</t>
+          <t>主人等级不足,还不能携带这只宝宝</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="0" t="inlineStr">
         <is>
-          <t>PetNoAutoPlan</t>
+          <t>PetAlreadyActive</t>
         </is>
       </c>
       <c r="B278" s="0" t="inlineStr">
         <is>
-          <t>没有可用的自动加点方案</t>
+          <t>这只宝宝已经在出战中</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="0" t="inlineStr">
         <is>
-          <t>PetNothingToChange</t>
+          <t>PetNotActive</t>
         </is>
       </c>
       <c r="B279" s="0" t="inlineStr">
         <is>
-          <t>宝宝属性没有变化</t>
+          <t>当前没有出战的宝宝</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="0" t="inlineStr">
         <is>
-          <t>PetIdGenerateFailed</t>
+          <t>PetSummonCooldown</t>
         </is>
       </c>
       <c r="B280" s="0" t="inlineStr">
         <is>
-          <t>宝宝创建失败,请稍后再试</t>
-        </is>
-      </c>
-      <c r="C280" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="281"/>
+          <t>操作太频繁,请稍后再试</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="0" t="inlineStr">
+        <is>
+          <t>PetNameInvalid</t>
+        </is>
+      </c>
+      <c r="B281" s="0" t="inlineStr">
+        <is>
+          <t>宝宝名称不合法</t>
+        </is>
+      </c>
+    </row>
     <row r="282">
       <c r="A282" s="0" t="inlineStr">
         <is>
-          <t>//asset_error base=27000 width=1000</t>
+          <t>PetInBattle</t>
+        </is>
+      </c>
+      <c r="B282" s="0" t="inlineStr">
+        <is>
+          <t>战斗中不能操作宝宝</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="0" t="inlineStr">
         <is>
-          <t>AssetCurrencyInsufficient</t>
+          <t>PetPointsNotEnough</t>
         </is>
       </c>
       <c r="B283" s="0" t="inlineStr">
         <is>
-          <t>货币不足</t>
+          <t>宝宝剩余点数不足</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="0" t="inlineStr">
         <is>
-          <t>AssetBagFull</t>
+          <t>PetPointsCannotDecrease</t>
         </is>
       </c>
       <c r="B284" s="0" t="inlineStr">
         <is>
-          <t>背包已满，请腾出空间，之后会重试发放；超过时限可能取消</t>
+          <t>已分配的点数不能减少,请使用洗点</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="0" t="inlineStr">
         <is>
-          <t>AssetInBattle</t>
+          <t>PetDimensionCapExceeded</t>
         </is>
       </c>
       <c r="B285" s="0" t="inlineStr">
         <is>
-          <t>战斗中暂不结算，稍后自动重试；超过时限可能取消</t>
+          <t>超过单项可分配上限</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="0" t="inlineStr">
         <is>
-          <t>AssetFrozen</t>
+          <t>PetDimensionNotFound</t>
         </is>
       </c>
       <c r="B286" s="0" t="inlineStr">
         <is>
-          <t>角色迁移中，稍后自动重试；超过时限可能取消</t>
+          <t>宝宝属性维度不存在</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="0" t="inlineStr">
         <is>
-          <t>AssetInvalidBundle</t>
+          <t>PetGoldNotEnough</t>
         </is>
       </c>
       <c r="B287" s="0" t="inlineStr">
         <is>
-          <t>资产指令无效</t>
-        </is>
-      </c>
-      <c r="C287" s="0" t="n">
-        <v>1</v>
+          <t>金币不足</t>
+        </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="0" t="inlineStr">
         <is>
-          <t>AssetBlocked</t>
+          <t>PetNoAutoPlan</t>
         </is>
       </c>
       <c r="B288" s="0" t="inlineStr">
         <is>
-          <t>该资产当前被禁止获取</t>
+          <t>没有可用的自动加点方案</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="0" t="inlineStr">
         <is>
-          <t>AssetPlayerNotHere</t>
+          <t>PetNothingToChange</t>
         </is>
       </c>
       <c r="B289" s="0" t="inlineStr">
         <is>
-          <t>角色不在线，上线后重试；超过时限可能取消</t>
+          <t>宝宝属性没有变化</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="0" t="inlineStr">
         <is>
-          <t>AssetPartialApplied</t>
+          <t>PetIdGenerateFailed</t>
         </is>
       </c>
       <c r="B290" s="0" t="inlineStr">
         <is>
-          <t>资产只发放了一部分，已记录，将由客服补偿</t>
+          <t>宝宝创建失败,请稍后再试</t>
         </is>
       </c>
       <c r="C290" s="0" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="291">
-      <c r="A291" s="0" t="inlineStr">
+    <row r="291"/>
+    <row r="292">
+      <c r="A292" s="0" t="inlineStr">
+        <is>
+          <t>//asset_error base=27000 width=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="0" t="inlineStr">
+        <is>
+          <t>AssetCurrencyInsufficient</t>
+        </is>
+      </c>
+      <c r="B293" s="0" t="inlineStr">
+        <is>
+          <t>货币不足</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="0" t="inlineStr">
+        <is>
+          <t>AssetBagFull</t>
+        </is>
+      </c>
+      <c r="B294" s="0" t="inlineStr">
+        <is>
+          <t>背包已满，请腾出空间，之后会重试发放；超过时限可能取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="0" t="inlineStr">
+        <is>
+          <t>AssetInBattle</t>
+        </is>
+      </c>
+      <c r="B295" s="0" t="inlineStr">
+        <is>
+          <t>战斗中暂不结算，稍后自动重试；超过时限可能取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="0" t="inlineStr">
+        <is>
+          <t>AssetFrozen</t>
+        </is>
+      </c>
+      <c r="B296" s="0" t="inlineStr">
+        <is>
+          <t>角色迁移中，稍后自动重试；超过时限可能取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="0" t="inlineStr">
+        <is>
+          <t>AssetInvalidBundle</t>
+        </is>
+      </c>
+      <c r="B297" s="0" t="inlineStr">
+        <is>
+          <t>资产指令无效</t>
+        </is>
+      </c>
+      <c r="C297" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="0" t="inlineStr">
+        <is>
+          <t>AssetBlocked</t>
+        </is>
+      </c>
+      <c r="B298" s="0" t="inlineStr">
+        <is>
+          <t>该资产当前被禁止获取</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="0" t="inlineStr">
+        <is>
+          <t>AssetPlayerNotHere</t>
+        </is>
+      </c>
+      <c r="B299" s="0" t="inlineStr">
+        <is>
+          <t>角色不在线，上线后重试；超过时限可能取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="0" t="inlineStr">
+        <is>
+          <t>AssetPartialApplied</t>
+        </is>
+      </c>
+      <c r="B300" s="0" t="inlineStr">
+        <is>
+          <t>资产只发放了一部分，已记录，将由客服补偿</t>
+        </is>
+      </c>
+      <c r="C300" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="0" t="inlineStr">
         <is>
           <t>AssetAuthFailed</t>
         </is>
       </c>
-      <c r="B291" s="0" t="inlineStr">
+      <c r="B301" s="0" t="inlineStr">
         <is>
           <t>资产指令校验失败</t>
         </is>
       </c>
-      <c r="C291" s="0" t="n">
+      <c r="C301" s="0" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>